<commit_message>
minor template writer update
</commit_message>
<xml_diff>
--- a/data/Financial Spreadsheet Template v2.xlsx
+++ b/data/Financial Spreadsheet Template v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfizer-my.sharepoint.com/personal/hoveyo_pfizer_com/Documents/financial-automation-project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="621" documentId="8_{ADF84F62-CC85-48F6-A2B9-288B99318624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AE2532D-A34C-411F-9EC1-825B7644D982}"/>
+  <xr:revisionPtr revIDLastSave="631" documentId="8_{ADF84F62-CC85-48F6-A2B9-288B99318624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5A7AF0B-2BF2-4B61-9C9A-5B6EDF1F667E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="12480" tabRatio="590" xr2:uid="{0996C49B-04E6-42AE-AA83-2F64BE89A626}"/>
   </bookViews>
@@ -1185,7 +1185,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="142">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1307,7 +1307,6 @@
     <xf numFmtId="3" fontId="0" fillId="5" borderId="33" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1375,15 +1374,6 @@
     <xf numFmtId="3" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1402,6 +1392,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency 2" xfId="2" xr:uid="{C819F491-96B6-415F-B3EE-ED5A59A1E95E}"/>
@@ -1410,6 +1409,13 @@
     <cellStyle name="Normal 2 2" xfId="3" xr:uid="{EFDA3BDD-7E2C-4F3B-BEB7-091BB23895D4}"/>
   </cellStyles>
   <dxfs count="9">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF7C80"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1456,13 +1462,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1836,9 +1835,9 @@
         <v>92</v>
       </c>
       <c r="E3" s="7">
-        <v>2024</v>
-      </c>
-      <c r="F3" s="128">
+        <v>2025</v>
+      </c>
+      <c r="F3" s="127">
         <f>C3</f>
         <v>0</v>
       </c>
@@ -1860,9 +1859,9 @@
         <v>2351818</v>
       </c>
       <c r="E4" s="7">
-        <v>2024</v>
-      </c>
-      <c r="F4" s="128">
+        <v>2025</v>
+      </c>
+      <c r="F4" s="127">
         <v>0</v>
       </c>
     </row>
@@ -1874,7 +1873,7 @@
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
-      <c r="F5" s="129"/>
+      <c r="F5" s="128"/>
     </row>
     <row r="6" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
@@ -1885,7 +1884,7 @@
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
-      <c r="E6" s="113" t="str">
+      <c r="E6" s="112" t="str">
         <f ca="1">IF(SUMIFS(BR:BR,A:A,"Contingency")&gt;0,"Contingency is "&amp;TEXT(SUMIFS(BR:BR,A:A,"Contingency"),"$#,##"),IF(SUMIFS(BR:BR,A:A,"Contingency")&lt;0,"Overspent by "&amp;TEXT(SUMIFS(BR:BR,A:A,"Contingency"),"$#,##"),"No contingency"))</f>
         <v>No contingency</v>
       </c>
@@ -1893,9 +1892,9 @@
     </row>
     <row r="7" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A7" s="13"/>
-      <c r="B7" s="112"/>
-      <c r="C7" s="111"/>
-      <c r="D7" s="111"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="110"/>
+      <c r="D7" s="110"/>
       <c r="E7" s="14"/>
       <c r="F7" s="15"/>
       <c r="O7" s="16"/>
@@ -1911,158 +1910,158 @@
         <f>C4-BR13</f>
         <v>0</v>
       </c>
-      <c r="D9" s="114"/>
-      <c r="E9" s="120" t="s">
+      <c r="D9" s="113"/>
+      <c r="E9" s="119" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="120" t="s">
+      <c r="F9" s="119" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="121" t="s">
+      <c r="G9" s="120" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="126" t="s">
+      <c r="A10" s="125" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="127" t="e">
+      <c r="B10" s="126" t="e">
         <f>B9/C4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D10" s="122" t="s">
+      <c r="D10" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="115"/>
-      <c r="F10" s="115"/>
-      <c r="G10" s="116"/>
+      <c r="E10" s="114"/>
+      <c r="F10" s="114"/>
+      <c r="G10" s="115"/>
       <c r="BS10" s="67" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:73" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="124" t="s">
+      <c r="A11" s="123" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="125">
+      <c r="B11" s="124">
         <f ca="1">SUMIFS(J12:BQ12,J13:BQ13,"&lt;="&amp;TODAY())</f>
         <v>0</v>
       </c>
-      <c r="D11" s="122" t="s">
+      <c r="D11" s="121" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="115">
+      <c r="E11" s="114">
         <f ca="1">SUM(J11:X11,Y12:AM12)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="115">
+      <c r="F11" s="114">
         <f ca="1">SUM(AN12:BQ12)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="116">
+      <c r="G11" s="115">
         <f ca="1">SUM(J11:X11,Y12:BQ12)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="136" t="s">
+      <c r="H11" s="132" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="137"/>
-      <c r="J11" s="130" cm="1">
+      <c r="I11" s="133"/>
+      <c r="J11" s="129" cm="1">
         <f t="array" aca="1" ref="J11" ca="1">SUM(M15:M25)+SUM(_xlfn._xlws.FILTER(L15:L25,M15:M25=""))+SUM(_xlfn._xlws.FILTER(K15:K25,(L15:L25="")*(M15:M25="")))+SUMIFS(N15:N25,M15:M25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(J15:J25)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="131"/>
-      <c r="L11" s="131"/>
-      <c r="M11" s="131"/>
-      <c r="N11" s="132"/>
-      <c r="O11" s="130" cm="1">
+      <c r="K11" s="130"/>
+      <c r="L11" s="130"/>
+      <c r="M11" s="130"/>
+      <c r="N11" s="131"/>
+      <c r="O11" s="129" cm="1">
         <f t="array" aca="1" ref="O11" ca="1">SUM(R15:R25)+SUM(_xlfn._xlws.FILTER(Q15:Q25,R15:R25=""))+SUM(_xlfn._xlws.FILTER(P15:P25,(Q15:Q25="")*(R15:R25="")))+SUMIFS(S15:S25,R15:R25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(O15:O25)</f>
         <v>0</v>
       </c>
-      <c r="P11" s="131"/>
-      <c r="Q11" s="131"/>
-      <c r="R11" s="131"/>
-      <c r="S11" s="132"/>
-      <c r="T11" s="130" cm="1">
+      <c r="P11" s="130"/>
+      <c r="Q11" s="130"/>
+      <c r="R11" s="130"/>
+      <c r="S11" s="131"/>
+      <c r="T11" s="129" cm="1">
         <f t="array" aca="1" ref="T11" ca="1">SUM(W15:W25)+SUM(_xlfn._xlws.FILTER(V15:V25,W15:W25=""))+SUM(_xlfn._xlws.FILTER(U15:U25,(V15:V25="")*(W15:W25="")))+SUMIFS(X15:X25,W15:W25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(T15:T25)</f>
         <v>0</v>
       </c>
-      <c r="U11" s="131"/>
-      <c r="V11" s="131"/>
-      <c r="W11" s="131"/>
-      <c r="X11" s="132"/>
-      <c r="Y11" s="130" cm="1">
+      <c r="U11" s="130"/>
+      <c r="V11" s="130"/>
+      <c r="W11" s="130"/>
+      <c r="X11" s="131"/>
+      <c r="Y11" s="129" cm="1">
         <f t="array" aca="1" ref="Y11" ca="1">SUM(AB15:AB25)+SUM(_xlfn._xlws.FILTER(AA15:AA25,AB15:AB25=""))+SUM(_xlfn._xlws.FILTER(Z15:Z25,(AA15:AA25="")*(AB15:AB25="")))+SUMIFS(AC15:AC25,AB15:AB25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(Y15:Y25)</f>
         <v>0</v>
       </c>
-      <c r="Z11" s="131"/>
-      <c r="AA11" s="131"/>
-      <c r="AB11" s="131"/>
-      <c r="AC11" s="132"/>
-      <c r="AD11" s="130" cm="1">
+      <c r="Z11" s="130"/>
+      <c r="AA11" s="130"/>
+      <c r="AB11" s="130"/>
+      <c r="AC11" s="131"/>
+      <c r="AD11" s="129" cm="1">
         <f t="array" aca="1" ref="AD11" ca="1">SUM(AG15:AG25)+SUM(_xlfn._xlws.FILTER(AF15:AF25,AG15:AG25=""))+SUM(_xlfn._xlws.FILTER(AE15:AE25,(AF15:AF25="")*(AG15:AG25="")))+SUMIFS(AH15:AH25,AG15:AG25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AD15:AD25)</f>
         <v>0</v>
       </c>
-      <c r="AE11" s="131"/>
-      <c r="AF11" s="131"/>
-      <c r="AG11" s="131"/>
-      <c r="AH11" s="132"/>
-      <c r="AI11" s="130" cm="1">
+      <c r="AE11" s="130"/>
+      <c r="AF11" s="130"/>
+      <c r="AG11" s="130"/>
+      <c r="AH11" s="131"/>
+      <c r="AI11" s="129" cm="1">
         <f t="array" aca="1" ref="AI11" ca="1">SUM(AL15:AL25)+SUM(_xlfn._xlws.FILTER(AK15:AK25,AL15:AL25=""))+SUM(_xlfn._xlws.FILTER(AJ15:AJ25,(AK15:AK25="")*(AL15:AL25="")))+SUMIFS(AM15:AM25,AL15:AL25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AI15:AI25)</f>
         <v>0</v>
       </c>
-      <c r="AJ11" s="131"/>
-      <c r="AK11" s="131"/>
-      <c r="AL11" s="131"/>
-      <c r="AM11" s="132"/>
-      <c r="AN11" s="130" cm="1">
+      <c r="AJ11" s="130"/>
+      <c r="AK11" s="130"/>
+      <c r="AL11" s="130"/>
+      <c r="AM11" s="131"/>
+      <c r="AN11" s="129" cm="1">
         <f t="array" aca="1" ref="AN11" ca="1">SUM(AQ15:AQ25)+SUM(_xlfn._xlws.FILTER(AP15:AP25,AQ15:AQ25=""))+SUM(_xlfn._xlws.FILTER(AO15:AO25,(AP15:AP25="")*(AQ15:AQ25="")))+SUMIFS(AR15:AR25,AQ15:AQ25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AN15:AN25)</f>
         <v>0</v>
       </c>
-      <c r="AO11" s="131"/>
-      <c r="AP11" s="131"/>
-      <c r="AQ11" s="131"/>
-      <c r="AR11" s="132"/>
-      <c r="AS11" s="130" cm="1">
+      <c r="AO11" s="130"/>
+      <c r="AP11" s="130"/>
+      <c r="AQ11" s="130"/>
+      <c r="AR11" s="131"/>
+      <c r="AS11" s="129" cm="1">
         <f t="array" aca="1" ref="AS11" ca="1">SUM(AV15:AV25)+SUM(_xlfn._xlws.FILTER(AU15:AU25,AV15:AV25=""))+SUM(_xlfn._xlws.FILTER(AT15:AT25,(AU15:AU25="")*(AV15:AV25="")))+SUMIFS(AW15:AW25,AV15:AV25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AS15:AS25)</f>
         <v>0</v>
       </c>
-      <c r="AT11" s="131"/>
-      <c r="AU11" s="131"/>
-      <c r="AV11" s="131"/>
-      <c r="AW11" s="132"/>
-      <c r="AX11" s="130" cm="1">
+      <c r="AT11" s="130"/>
+      <c r="AU11" s="130"/>
+      <c r="AV11" s="130"/>
+      <c r="AW11" s="131"/>
+      <c r="AX11" s="129" cm="1">
         <f t="array" aca="1" ref="AX11" ca="1">SUM(BA15:BA25)+SUM(_xlfn._xlws.FILTER(AZ15:AZ25,BA15:BA25=""))+SUM(_xlfn._xlws.FILTER(AY15:AY25,(AZ15:AZ25="")*(BA15:BA25="")))+SUMIFS(BB15:BB25,BA15:BA25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AX15:AX25)</f>
         <v>0</v>
       </c>
-      <c r="AY11" s="131"/>
-      <c r="AZ11" s="131"/>
-      <c r="BA11" s="131"/>
-      <c r="BB11" s="132"/>
-      <c r="BC11" s="130" cm="1">
+      <c r="AY11" s="130"/>
+      <c r="AZ11" s="130"/>
+      <c r="BA11" s="130"/>
+      <c r="BB11" s="131"/>
+      <c r="BC11" s="129" cm="1">
         <f t="array" aca="1" ref="BC11" ca="1">SUM(BF15:BF25)+SUM(_xlfn._xlws.FILTER(BE15:BE25,BF15:BF25=""))+SUM(_xlfn._xlws.FILTER(BD15:BD25,(BE15:BE25="")*(BF15:BF25="")))+SUMIFS(BG15:BG25,BF15:BF25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(BC15:BC25)</f>
         <v>0</v>
       </c>
-      <c r="BD11" s="131"/>
-      <c r="BE11" s="131"/>
-      <c r="BF11" s="131"/>
-      <c r="BG11" s="132"/>
-      <c r="BH11" s="130" cm="1">
+      <c r="BD11" s="130"/>
+      <c r="BE11" s="130"/>
+      <c r="BF11" s="130"/>
+      <c r="BG11" s="131"/>
+      <c r="BH11" s="129" cm="1">
         <f t="array" aca="1" ref="BH11" ca="1">SUM(BK15:BK25)+SUM(_xlfn._xlws.FILTER(BJ15:BJ25,BK15:BK25=""))+SUM(_xlfn._xlws.FILTER(BI15:BI25,(BJ15:BJ25="")*(BK15:BK25="")))+SUMIFS(BL15:BL25,BK15:BK25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(BH15:BH25)</f>
         <v>0</v>
       </c>
-      <c r="BI11" s="131"/>
-      <c r="BJ11" s="131"/>
-      <c r="BK11" s="131"/>
-      <c r="BL11" s="132"/>
-      <c r="BM11" s="130" cm="1">
+      <c r="BI11" s="130"/>
+      <c r="BJ11" s="130"/>
+      <c r="BK11" s="130"/>
+      <c r="BL11" s="131"/>
+      <c r="BM11" s="129" cm="1">
         <f t="array" aca="1" ref="BM11" ca="1">SUM(BP15:BP25)+SUM(_xlfn._xlws.FILTER(BO15:BO25,BP15:BP25=""))+SUM(_xlfn._xlws.FILTER(BN15:BN25,(BO15:BO25="")*(BP15:BP25="")))+SUMIFS(BQ15:BQ25,BP15:BP25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(BM15:BM25)</f>
         <v>0</v>
       </c>
-      <c r="BN11" s="131"/>
-      <c r="BO11" s="131"/>
-      <c r="BP11" s="131"/>
-      <c r="BQ11" s="132"/>
+      <c r="BN11" s="130"/>
+      <c r="BO11" s="130"/>
+      <c r="BP11" s="130"/>
+      <c r="BQ11" s="131"/>
       <c r="BR11" s="21" t="s">
         <v>13</v>
       </c>
@@ -2075,125 +2074,125 @@
       <c r="A12" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="119">
+      <c r="B12" s="118">
         <f ca="1">C4-B11</f>
         <v>0</v>
       </c>
-      <c r="D12" s="123" t="s">
+      <c r="D12" s="122" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="117">
+      <c r="E12" s="116">
         <f ca="1">E11-E10</f>
         <v>0</v>
       </c>
-      <c r="F12" s="117">
+      <c r="F12" s="116">
         <f t="shared" ref="F12:G12" ca="1" si="0">F11-F10</f>
         <v>0</v>
       </c>
-      <c r="G12" s="118">
+      <c r="G12" s="117">
         <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="138" t="s">
+      <c r="H12" s="134" t="s">
         <v>16</v>
       </c>
-      <c r="I12" s="139"/>
-      <c r="J12" s="130" cm="1">
+      <c r="I12" s="135"/>
+      <c r="J12" s="129" cm="1">
         <f t="array" aca="1" ref="J12" ca="1">SUM(M15:M25)+SUM(_xlfn._xlws.FILTER(L15:L25,M15:M25=""))+SUM(_xlfn._xlws.FILTER(K15:K25,(L15:L25="")*(M15:M25="")))</f>
         <v>0</v>
       </c>
-      <c r="K12" s="131"/>
-      <c r="L12" s="131"/>
-      <c r="M12" s="131"/>
-      <c r="N12" s="132"/>
-      <c r="O12" s="130" cm="1">
+      <c r="K12" s="130"/>
+      <c r="L12" s="130"/>
+      <c r="M12" s="130"/>
+      <c r="N12" s="131"/>
+      <c r="O12" s="129" cm="1">
         <f t="array" aca="1" ref="O12" ca="1">SUM(R15:R25)+SUM(_xlfn._xlws.FILTER(Q15:Q25,R15:R25=""))+SUM(_xlfn._xlws.FILTER(P15:P25,(Q15:Q25="")*(R15:R25="")))</f>
         <v>0</v>
       </c>
-      <c r="P12" s="131"/>
-      <c r="Q12" s="131"/>
-      <c r="R12" s="131"/>
-      <c r="S12" s="132"/>
-      <c r="T12" s="130" cm="1">
+      <c r="P12" s="130"/>
+      <c r="Q12" s="130"/>
+      <c r="R12" s="130"/>
+      <c r="S12" s="131"/>
+      <c r="T12" s="129" cm="1">
         <f t="array" aca="1" ref="T12" ca="1">SUM(W15:W25)+SUM(_xlfn._xlws.FILTER(V15:V25,W15:W25=""))+SUM(_xlfn._xlws.FILTER(U15:U25,(V15:V25="")*(W15:W25="")))</f>
         <v>0</v>
       </c>
-      <c r="U12" s="131"/>
-      <c r="V12" s="131"/>
-      <c r="W12" s="131"/>
-      <c r="X12" s="132"/>
-      <c r="Y12" s="130" cm="1">
+      <c r="U12" s="130"/>
+      <c r="V12" s="130"/>
+      <c r="W12" s="130"/>
+      <c r="X12" s="131"/>
+      <c r="Y12" s="129" cm="1">
         <f t="array" aca="1" ref="Y12" ca="1">SUM(AB15:AB25)+SUM(_xlfn._xlws.FILTER(AA15:AA25,AB15:AB25=""))+SUM(_xlfn._xlws.FILTER(Z15:Z25,(AA15:AA25="")*(AB15:AB25="")))</f>
         <v>0</v>
       </c>
-      <c r="Z12" s="131"/>
-      <c r="AA12" s="131"/>
-      <c r="AB12" s="131"/>
-      <c r="AC12" s="132"/>
-      <c r="AD12" s="130" cm="1">
+      <c r="Z12" s="130"/>
+      <c r="AA12" s="130"/>
+      <c r="AB12" s="130"/>
+      <c r="AC12" s="131"/>
+      <c r="AD12" s="129" cm="1">
         <f t="array" aca="1" ref="AD12" ca="1">SUM(AG15:AG25)+SUM(_xlfn._xlws.FILTER(AF15:AF25,AG15:AG25=""))+SUM(_xlfn._xlws.FILTER(AE15:AE25,(AF15:AF25="")*(AG15:AG25="")))</f>
         <v>0</v>
       </c>
-      <c r="AE12" s="131"/>
-      <c r="AF12" s="131"/>
-      <c r="AG12" s="131"/>
-      <c r="AH12" s="132"/>
-      <c r="AI12" s="130" cm="1">
+      <c r="AE12" s="130"/>
+      <c r="AF12" s="130"/>
+      <c r="AG12" s="130"/>
+      <c r="AH12" s="131"/>
+      <c r="AI12" s="129" cm="1">
         <f t="array" aca="1" ref="AI12" ca="1">SUM(AL15:AL25)+SUM(_xlfn._xlws.FILTER(AK15:AK25,AL15:AL25=""))+SUM(_xlfn._xlws.FILTER(AJ15:AJ25,(AK15:AK25="")*(AL15:AL25="")))</f>
         <v>0</v>
       </c>
-      <c r="AJ12" s="131"/>
-      <c r="AK12" s="131"/>
-      <c r="AL12" s="131"/>
-      <c r="AM12" s="132"/>
-      <c r="AN12" s="130" cm="1">
+      <c r="AJ12" s="130"/>
+      <c r="AK12" s="130"/>
+      <c r="AL12" s="130"/>
+      <c r="AM12" s="131"/>
+      <c r="AN12" s="129" cm="1">
         <f t="array" aca="1" ref="AN12" ca="1">SUM(AQ15:AQ25)+SUM(_xlfn._xlws.FILTER(AP15:AP25,AQ15:AQ25=""))+SUM(_xlfn._xlws.FILTER(AO15:AO25,(AP15:AP25="")*(AQ15:AQ25="")))</f>
         <v>0</v>
       </c>
-      <c r="AO12" s="131"/>
-      <c r="AP12" s="131"/>
-      <c r="AQ12" s="131"/>
-      <c r="AR12" s="132"/>
-      <c r="AS12" s="130" cm="1">
+      <c r="AO12" s="130"/>
+      <c r="AP12" s="130"/>
+      <c r="AQ12" s="130"/>
+      <c r="AR12" s="131"/>
+      <c r="AS12" s="129" cm="1">
         <f t="array" aca="1" ref="AS12" ca="1">SUM(AV15:AV25)+SUM(_xlfn._xlws.FILTER(AU15:AU25,AV15:AV25=""))+SUM(_xlfn._xlws.FILTER(AT15:AT25,(AU15:AU25="")*(AV15:AV25="")))</f>
         <v>0</v>
       </c>
-      <c r="AT12" s="131"/>
-      <c r="AU12" s="131"/>
-      <c r="AV12" s="131"/>
-      <c r="AW12" s="132"/>
-      <c r="AX12" s="130" cm="1">
+      <c r="AT12" s="130"/>
+      <c r="AU12" s="130"/>
+      <c r="AV12" s="130"/>
+      <c r="AW12" s="131"/>
+      <c r="AX12" s="129" cm="1">
         <f t="array" aca="1" ref="AX12" ca="1">SUM(BA15:BA25)+SUM(_xlfn._xlws.FILTER(AZ15:AZ25,BA15:BA25=""))+SUM(_xlfn._xlws.FILTER(AY15:AY25,(AZ15:AZ25="")*(BA15:BA25="")))</f>
         <v>0</v>
       </c>
-      <c r="AY12" s="131"/>
-      <c r="AZ12" s="131"/>
-      <c r="BA12" s="131"/>
-      <c r="BB12" s="132"/>
-      <c r="BC12" s="130" cm="1">
+      <c r="AY12" s="130"/>
+      <c r="AZ12" s="130"/>
+      <c r="BA12" s="130"/>
+      <c r="BB12" s="131"/>
+      <c r="BC12" s="129" cm="1">
         <f t="array" aca="1" ref="BC12" ca="1">SUM(BF15:BF25)+SUM(_xlfn._xlws.FILTER(BE15:BE25,BF15:BF25=""))+SUM(_xlfn._xlws.FILTER(BD15:BD25,(BE15:BE25="")*(BF15:BF25="")))</f>
         <v>0</v>
       </c>
-      <c r="BD12" s="131"/>
-      <c r="BE12" s="131"/>
-      <c r="BF12" s="131"/>
-      <c r="BG12" s="132"/>
-      <c r="BH12" s="130" cm="1">
+      <c r="BD12" s="130"/>
+      <c r="BE12" s="130"/>
+      <c r="BF12" s="130"/>
+      <c r="BG12" s="131"/>
+      <c r="BH12" s="129" cm="1">
         <f t="array" aca="1" ref="BH12" ca="1">SUM(BK15:BK25)+SUM(_xlfn._xlws.FILTER(BJ15:BJ25,BK15:BK25=""))+SUM(_xlfn._xlws.FILTER(BI15:BI25,(BJ15:BJ25="")*(BK15:BK25="")))</f>
         <v>0</v>
       </c>
-      <c r="BI12" s="131"/>
-      <c r="BJ12" s="131"/>
-      <c r="BK12" s="131"/>
-      <c r="BL12" s="132"/>
-      <c r="BM12" s="130" cm="1">
+      <c r="BI12" s="130"/>
+      <c r="BJ12" s="130"/>
+      <c r="BK12" s="130"/>
+      <c r="BL12" s="131"/>
+      <c r="BM12" s="129" cm="1">
         <f t="array" aca="1" ref="BM12" ca="1">SUM(BP15:BP25)+SUM(_xlfn._xlws.FILTER(BO15:BO25,BP15:BP25=""))+SUM(_xlfn._xlws.FILTER(BN15:BN25,(BO15:BO25="")*(BP15:BP25="")))</f>
         <v>0</v>
       </c>
-      <c r="BN12" s="131"/>
-      <c r="BO12" s="131"/>
-      <c r="BP12" s="131"/>
-      <c r="BQ12" s="132"/>
+      <c r="BN12" s="130"/>
+      <c r="BO12" s="130"/>
+      <c r="BP12" s="130"/>
+      <c r="BQ12" s="131"/>
       <c r="BR12" s="21"/>
       <c r="BS12" s="22"/>
     </row>
@@ -2201,116 +2200,116 @@
       <c r="A13" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="140" t="s">
+      <c r="H13" s="136" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="141"/>
-      <c r="J13" s="133">
+      <c r="I13" s="137"/>
+      <c r="J13" s="138">
         <v>45688</v>
       </c>
-      <c r="K13" s="134" t="s">
+      <c r="K13" s="139" t="s">
         <v>19</v>
       </c>
-      <c r="L13" s="134"/>
-      <c r="M13" s="134"/>
-      <c r="N13" s="134"/>
-      <c r="O13" s="133" t="s">
+      <c r="L13" s="139"/>
+      <c r="M13" s="139"/>
+      <c r="N13" s="139"/>
+      <c r="O13" s="138" t="s">
         <v>97</v>
       </c>
-      <c r="P13" s="134"/>
-      <c r="Q13" s="134"/>
-      <c r="R13" s="134"/>
-      <c r="S13" s="135"/>
-      <c r="T13" s="133">
+      <c r="P13" s="139"/>
+      <c r="Q13" s="139"/>
+      <c r="R13" s="139"/>
+      <c r="S13" s="140"/>
+      <c r="T13" s="138">
         <v>45747</v>
       </c>
-      <c r="U13" s="134" t="s">
+      <c r="U13" s="139" t="s">
         <v>20</v>
       </c>
-      <c r="V13" s="134"/>
-      <c r="W13" s="134"/>
-      <c r="X13" s="135"/>
-      <c r="Y13" s="133">
+      <c r="V13" s="139"/>
+      <c r="W13" s="139"/>
+      <c r="X13" s="140"/>
+      <c r="Y13" s="138">
         <v>45777</v>
       </c>
-      <c r="Z13" s="134" t="s">
+      <c r="Z13" s="139" t="s">
         <v>21</v>
       </c>
-      <c r="AA13" s="134"/>
-      <c r="AB13" s="134"/>
-      <c r="AC13" s="135"/>
-      <c r="AD13" s="133">
+      <c r="AA13" s="139"/>
+      <c r="AB13" s="139"/>
+      <c r="AC13" s="140"/>
+      <c r="AD13" s="138">
         <v>45808</v>
       </c>
-      <c r="AE13" s="134" t="s">
+      <c r="AE13" s="139" t="s">
         <v>22</v>
       </c>
-      <c r="AF13" s="134"/>
-      <c r="AG13" s="134"/>
-      <c r="AH13" s="135"/>
-      <c r="AI13" s="133">
+      <c r="AF13" s="139"/>
+      <c r="AG13" s="139"/>
+      <c r="AH13" s="140"/>
+      <c r="AI13" s="138">
         <v>45838</v>
       </c>
-      <c r="AJ13" s="134" t="s">
+      <c r="AJ13" s="139" t="s">
         <v>23</v>
       </c>
-      <c r="AK13" s="134"/>
-      <c r="AL13" s="134"/>
-      <c r="AM13" s="135"/>
-      <c r="AN13" s="133">
+      <c r="AK13" s="139"/>
+      <c r="AL13" s="139"/>
+      <c r="AM13" s="140"/>
+      <c r="AN13" s="138">
         <v>45869</v>
       </c>
-      <c r="AO13" s="134" t="s">
+      <c r="AO13" s="139" t="s">
         <v>24</v>
       </c>
-      <c r="AP13" s="134"/>
-      <c r="AQ13" s="134"/>
-      <c r="AR13" s="135"/>
-      <c r="AS13" s="133">
+      <c r="AP13" s="139"/>
+      <c r="AQ13" s="139"/>
+      <c r="AR13" s="140"/>
+      <c r="AS13" s="138">
         <v>45900</v>
       </c>
-      <c r="AT13" s="134" t="s">
+      <c r="AT13" s="139" t="s">
         <v>25</v>
       </c>
-      <c r="AU13" s="134"/>
-      <c r="AV13" s="134"/>
-      <c r="AW13" s="135"/>
-      <c r="AX13" s="133">
+      <c r="AU13" s="139"/>
+      <c r="AV13" s="139"/>
+      <c r="AW13" s="140"/>
+      <c r="AX13" s="138">
         <v>45930</v>
       </c>
-      <c r="AY13" s="134" t="s">
+      <c r="AY13" s="139" t="s">
         <v>26</v>
       </c>
-      <c r="AZ13" s="134"/>
-      <c r="BA13" s="134"/>
-      <c r="BB13" s="135"/>
-      <c r="BC13" s="133">
+      <c r="AZ13" s="139"/>
+      <c r="BA13" s="139"/>
+      <c r="BB13" s="140"/>
+      <c r="BC13" s="138">
         <v>45961</v>
       </c>
-      <c r="BD13" s="134" t="s">
+      <c r="BD13" s="139" t="s">
         <v>27</v>
       </c>
-      <c r="BE13" s="134"/>
-      <c r="BF13" s="134"/>
-      <c r="BG13" s="135"/>
-      <c r="BH13" s="133">
+      <c r="BE13" s="139"/>
+      <c r="BF13" s="139"/>
+      <c r="BG13" s="140"/>
+      <c r="BH13" s="138">
         <v>45991</v>
       </c>
-      <c r="BI13" s="134" t="s">
+      <c r="BI13" s="139" t="s">
         <v>28</v>
       </c>
-      <c r="BJ13" s="134"/>
-      <c r="BK13" s="134"/>
-      <c r="BL13" s="135"/>
-      <c r="BM13" s="133">
+      <c r="BJ13" s="139"/>
+      <c r="BK13" s="139"/>
+      <c r="BL13" s="140"/>
+      <c r="BM13" s="138">
         <v>46022</v>
       </c>
-      <c r="BN13" s="134" t="s">
+      <c r="BN13" s="139" t="s">
         <v>29</v>
       </c>
-      <c r="BO13" s="134"/>
-      <c r="BP13" s="134"/>
-      <c r="BQ13" s="135"/>
+      <c r="BO13" s="139"/>
+      <c r="BP13" s="139"/>
+      <c r="BQ13" s="140"/>
       <c r="BR13" s="24">
         <f>SUM(BR15:BR24)</f>
         <v>0</v>
@@ -3287,116 +3286,122 @@
       <c r="BS21" s="73"/>
       <c r="BT21" s="74"/>
     </row>
-    <row r="22" spans="1:72" s="67" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="100" t="s">
+    <row r="22" spans="1:72" x14ac:dyDescent="0.25">
+      <c r="A22" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="B22" s="101"/>
-      <c r="C22" s="102"/>
-      <c r="D22" s="102"/>
-      <c r="E22" s="101"/>
-      <c r="F22" s="101"/>
-      <c r="G22" s="103"/>
-      <c r="H22" s="101"/>
-      <c r="I22" s="104"/>
-      <c r="J22" s="105"/>
-      <c r="K22" s="103"/>
-      <c r="L22" s="103"/>
-      <c r="M22" s="106"/>
-      <c r="N22" s="106" t="str">
+      <c r="B22" s="100"/>
+      <c r="C22" s="101"/>
+      <c r="D22" s="101"/>
+      <c r="E22" s="100"/>
+      <c r="F22" s="100"/>
+      <c r="G22" s="102"/>
+      <c r="H22" s="100"/>
+      <c r="I22" s="103"/>
+      <c r="J22" s="104"/>
+      <c r="K22" s="102"/>
+      <c r="L22" s="102"/>
+      <c r="M22" s="105"/>
+      <c r="N22" s="105" t="str">
         <f>IF(OR(L22="",M22=""),"",L22-M22)</f>
         <v/>
       </c>
-      <c r="O22" s="105"/>
-      <c r="P22" s="103"/>
-      <c r="Q22" s="103"/>
-      <c r="R22" s="106"/>
-      <c r="S22" s="107"/>
-      <c r="T22" s="108"/>
-      <c r="U22" s="103"/>
-      <c r="V22" s="103"/>
-      <c r="W22" s="106"/>
-      <c r="X22" s="107"/>
-      <c r="Y22" s="108"/>
-      <c r="Z22" s="103"/>
-      <c r="AA22" s="103"/>
-      <c r="AB22" s="106"/>
-      <c r="AC22" s="107" t="str">
-        <f t="shared" ref="AC22:AC24" si="14">IF(OR(AA22="",AB22=""),"",AA22-AB22)</f>
+      <c r="O22" s="104"/>
+      <c r="P22" s="102"/>
+      <c r="Q22" s="102"/>
+      <c r="R22" s="105"/>
+      <c r="S22" s="106" t="str">
+        <f t="shared" ref="S22:S24" si="14">IF(OR(Q22="",R22=""),"",Q22-R22)</f>
         <v/>
       </c>
-      <c r="AD22" s="108"/>
-      <c r="AE22" s="103"/>
-      <c r="AF22" s="103"/>
-      <c r="AG22" s="106"/>
-      <c r="AH22" s="107" t="str">
-        <f t="shared" ref="AH22:AH24" si="15">IF(OR(AF22="",AG22=""),"",AF22-AG22)</f>
+      <c r="T22" s="107"/>
+      <c r="U22" s="102"/>
+      <c r="V22" s="102"/>
+      <c r="W22" s="105"/>
+      <c r="X22" s="106" t="str">
+        <f t="shared" ref="X22:X24" si="15">IF(OR(V22="",W22=""),"",V22-W22)</f>
         <v/>
       </c>
-      <c r="AI22" s="108"/>
-      <c r="AJ22" s="103"/>
-      <c r="AK22" s="103"/>
-      <c r="AL22" s="106"/>
-      <c r="AM22" s="107" t="str">
-        <f t="shared" ref="AM22:AM24" si="16">IF(OR(AK22="",AL22=""),"",AK22-AL22)</f>
+      <c r="Y22" s="107"/>
+      <c r="Z22" s="102"/>
+      <c r="AA22" s="102"/>
+      <c r="AB22" s="105"/>
+      <c r="AC22" s="106" t="str">
+        <f t="shared" ref="AC22:AC24" si="16">IF(OR(AA22="",AB22=""),"",AA22-AB22)</f>
         <v/>
       </c>
-      <c r="AN22" s="108"/>
-      <c r="AO22" s="103"/>
-      <c r="AP22" s="103"/>
-      <c r="AQ22" s="106"/>
-      <c r="AR22" s="107" t="str">
-        <f t="shared" ref="AR22:AR24" si="17">IF(OR(AP22="",AQ22=""),"",AP22-AQ22)</f>
+      <c r="AD22" s="107"/>
+      <c r="AE22" s="102"/>
+      <c r="AF22" s="102"/>
+      <c r="AG22" s="105"/>
+      <c r="AH22" s="106" t="str">
+        <f t="shared" ref="AH22:AH24" si="17">IF(OR(AF22="",AG22=""),"",AF22-AG22)</f>
         <v/>
       </c>
-      <c r="AS22" s="108"/>
-      <c r="AT22" s="103"/>
-      <c r="AU22" s="103"/>
-      <c r="AV22" s="106"/>
-      <c r="AW22" s="107" t="str">
-        <f t="shared" ref="AW22:AW24" si="18">IF(OR(AU22="",AV22=""),"",AU22-AV22)</f>
+      <c r="AI22" s="107"/>
+      <c r="AJ22" s="102"/>
+      <c r="AK22" s="102"/>
+      <c r="AL22" s="105"/>
+      <c r="AM22" s="106" t="str">
+        <f t="shared" ref="AM22:AM24" si="18">IF(OR(AK22="",AL22=""),"",AK22-AL22)</f>
         <v/>
       </c>
-      <c r="AX22" s="108"/>
-      <c r="AY22" s="103"/>
-      <c r="AZ22" s="103"/>
-      <c r="BA22" s="106"/>
-      <c r="BB22" s="107" t="str">
-        <f t="shared" ref="BB22:BB24" si="19">IF(OR(AZ22="",BA22=""),"",AZ22-BA22)</f>
+      <c r="AN22" s="107"/>
+      <c r="AO22" s="102"/>
+      <c r="AP22" s="102"/>
+      <c r="AQ22" s="105"/>
+      <c r="AR22" s="106" t="str">
+        <f t="shared" ref="AR22:AR24" si="19">IF(OR(AP22="",AQ22=""),"",AP22-AQ22)</f>
         <v/>
       </c>
-      <c r="BC22" s="108"/>
-      <c r="BD22" s="103"/>
-      <c r="BE22" s="103"/>
-      <c r="BF22" s="106"/>
-      <c r="BG22" s="107" t="str">
-        <f t="shared" ref="BG22:BG24" si="20">IF(OR(BE22="",BF22=""),"",BE22-BF22)</f>
+      <c r="AS22" s="107"/>
+      <c r="AT22" s="102"/>
+      <c r="AU22" s="102"/>
+      <c r="AV22" s="105"/>
+      <c r="AW22" s="106" t="str">
+        <f t="shared" ref="AW22:AW24" si="20">IF(OR(AU22="",AV22=""),"",AU22-AV22)</f>
         <v/>
       </c>
-      <c r="BH22" s="108"/>
-      <c r="BI22" s="103"/>
-      <c r="BJ22" s="103"/>
-      <c r="BK22" s="106"/>
-      <c r="BL22" s="107" t="str">
-        <f t="shared" ref="BL22:BL24" si="21">IF(OR(BJ22="",BK22=""),"",BJ22-BK22)</f>
+      <c r="AX22" s="107"/>
+      <c r="AY22" s="102"/>
+      <c r="AZ22" s="102"/>
+      <c r="BA22" s="105"/>
+      <c r="BB22" s="106" t="str">
+        <f t="shared" ref="BB22:BB24" si="21">IF(OR(AZ22="",BA22=""),"",AZ22-BA22)</f>
         <v/>
       </c>
-      <c r="BM22" s="108"/>
-      <c r="BN22" s="103"/>
-      <c r="BO22" s="103"/>
-      <c r="BP22" s="106"/>
-      <c r="BQ22" s="107" t="str">
-        <f t="shared" ref="BQ22:BQ24" si="22">IF(OR(BO22="",BP22=""),"",BO22-BP22)</f>
+      <c r="BC22" s="107"/>
+      <c r="BD22" s="102"/>
+      <c r="BE22" s="102"/>
+      <c r="BF22" s="105"/>
+      <c r="BG22" s="106" t="str">
+        <f t="shared" ref="BG22:BG24" si="22">IF(OR(BE22="",BF22=""),"",BE22-BF22)</f>
         <v/>
       </c>
-      <c r="BR22" s="105">
+      <c r="BH22" s="107"/>
+      <c r="BI22" s="102"/>
+      <c r="BJ22" s="102"/>
+      <c r="BK22" s="105"/>
+      <c r="BL22" s="106" t="str">
+        <f t="shared" ref="BL22:BL24" si="23">IF(OR(BJ22="",BK22=""),"",BJ22-BK22)</f>
+        <v/>
+      </c>
+      <c r="BM22" s="107"/>
+      <c r="BN22" s="102"/>
+      <c r="BO22" s="102"/>
+      <c r="BP22" s="105"/>
+      <c r="BQ22" s="106" t="str">
+        <f t="shared" ref="BQ22:BQ24" si="24">IF(OR(BO22="",BP22=""),"",BO22-BP22)</f>
+        <v/>
+      </c>
+      <c r="BR22" s="104">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="BS22" s="109"/>
-      <c r="BT22" s="110"/>
+      <c r="BS22" s="108"/>
+      <c r="BT22" s="109"/>
     </row>
-    <row r="23" spans="1:72" s="87" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A23" s="76" t="s">
         <v>91</v>
       </c>
@@ -3423,7 +3428,7 @@
       <c r="Q23" s="81"/>
       <c r="R23" s="82"/>
       <c r="S23" s="83" t="str">
-        <f t="shared" ref="S22:S24" si="23">IF(OR(Q23="",R23=""),"",Q23-R23)</f>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="T23" s="84"/>
@@ -3431,7 +3436,7 @@
       <c r="V23" s="81"/>
       <c r="W23" s="82"/>
       <c r="X23" s="83" t="str">
-        <f t="shared" ref="X23:X24" si="24">IF(OR(V23="",W23=""),"",V23-W23)</f>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="Y23" s="84"/>
@@ -3439,7 +3444,7 @@
       <c r="AA23" s="81"/>
       <c r="AB23" s="82"/>
       <c r="AC23" s="83" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="AD23" s="84"/>
@@ -3447,7 +3452,7 @@
       <c r="AF23" s="81"/>
       <c r="AG23" s="82"/>
       <c r="AH23" s="83" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="AI23" s="84"/>
@@ -3455,7 +3460,7 @@
       <c r="AK23" s="81"/>
       <c r="AL23" s="82"/>
       <c r="AM23" s="83" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="AN23" s="84"/>
@@ -3463,7 +3468,7 @@
       <c r="AP23" s="81"/>
       <c r="AQ23" s="82"/>
       <c r="AR23" s="83" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="AS23" s="84"/>
@@ -3471,7 +3476,7 @@
       <c r="AU23" s="81"/>
       <c r="AV23" s="82"/>
       <c r="AW23" s="83" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="AX23" s="84"/>
@@ -3479,7 +3484,7 @@
       <c r="AZ23" s="81"/>
       <c r="BA23" s="82"/>
       <c r="BB23" s="83" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="BC23" s="84"/>
@@ -3487,7 +3492,7 @@
       <c r="BE23" s="81"/>
       <c r="BF23" s="82"/>
       <c r="BG23" s="83" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="BH23" s="84"/>
@@ -3495,7 +3500,7 @@
       <c r="BJ23" s="81"/>
       <c r="BK23" s="82"/>
       <c r="BL23" s="83" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
       <c r="BM23" s="84"/>
@@ -3503,7 +3508,7 @@
       <c r="BO23" s="81"/>
       <c r="BP23" s="82"/>
       <c r="BQ23" s="83" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="BR23" s="80">
@@ -3514,117 +3519,117 @@
       <c r="BT23" s="86"/>
     </row>
     <row r="24" spans="1:72" x14ac:dyDescent="0.25">
-      <c r="A24" s="88"/>
-      <c r="B24" s="89"/>
-      <c r="C24" s="90"/>
-      <c r="D24" s="90"/>
-      <c r="E24" s="89"/>
-      <c r="F24" s="89"/>
-      <c r="G24" s="89"/>
-      <c r="H24" s="89"/>
-      <c r="I24" s="91"/>
-      <c r="J24" s="92"/>
-      <c r="K24" s="93"/>
-      <c r="L24" s="93"/>
+      <c r="A24" s="87"/>
+      <c r="B24" s="88"/>
+      <c r="C24" s="89"/>
+      <c r="D24" s="89"/>
+      <c r="E24" s="88"/>
+      <c r="F24" s="88"/>
+      <c r="G24" s="88"/>
+      <c r="H24" s="88"/>
+      <c r="I24" s="90"/>
+      <c r="J24" s="91"/>
+      <c r="K24" s="92"/>
+      <c r="L24" s="92"/>
       <c r="M24" s="52"/>
       <c r="N24" s="52" t="str">
         <f t="shared" ref="N24:N25" si="25">IF(OR(L24="",M24=""),"",L24-M24)</f>
         <v/>
       </c>
-      <c r="O24" s="92"/>
-      <c r="P24" s="93"/>
-      <c r="Q24" s="93"/>
+      <c r="O24" s="91"/>
+      <c r="P24" s="92"/>
+      <c r="Q24" s="92"/>
       <c r="R24" s="52"/>
       <c r="S24" s="53" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="T24" s="58"/>
+      <c r="U24" s="92"/>
+      <c r="V24" s="92"/>
+      <c r="W24" s="52"/>
+      <c r="X24" s="53" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
+      <c r="Y24" s="58"/>
+      <c r="Z24" s="92"/>
+      <c r="AA24" s="92"/>
+      <c r="AB24" s="52"/>
+      <c r="AC24" s="53" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="AD24" s="58"/>
+      <c r="AE24" s="92"/>
+      <c r="AF24" s="92"/>
+      <c r="AG24" s="52"/>
+      <c r="AH24" s="53" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="AI24" s="58"/>
+      <c r="AJ24" s="92"/>
+      <c r="AK24" s="92"/>
+      <c r="AL24" s="52"/>
+      <c r="AM24" s="53" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="AN24" s="58"/>
+      <c r="AO24" s="92"/>
+      <c r="AP24" s="92"/>
+      <c r="AQ24" s="52"/>
+      <c r="AR24" s="53" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="AS24" s="58"/>
+      <c r="AT24" s="92"/>
+      <c r="AU24" s="92"/>
+      <c r="AV24" s="52"/>
+      <c r="AW24" s="53" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="AX24" s="58"/>
+      <c r="AY24" s="92"/>
+      <c r="AZ24" s="92"/>
+      <c r="BA24" s="52"/>
+      <c r="BB24" s="53" t="str">
+        <f t="shared" si="21"/>
+        <v/>
+      </c>
+      <c r="BC24" s="58"/>
+      <c r="BD24" s="92"/>
+      <c r="BE24" s="92"/>
+      <c r="BF24" s="52"/>
+      <c r="BG24" s="53" t="str">
+        <f t="shared" si="22"/>
+        <v/>
+      </c>
+      <c r="BH24" s="58"/>
+      <c r="BI24" s="92"/>
+      <c r="BJ24" s="92"/>
+      <c r="BK24" s="52"/>
+      <c r="BL24" s="53" t="str">
         <f t="shared" si="23"/>
         <v/>
       </c>
-      <c r="T24" s="58"/>
-      <c r="U24" s="93"/>
-      <c r="V24" s="93"/>
-      <c r="W24" s="52"/>
-      <c r="X24" s="53" t="str">
+      <c r="BM24" s="58"/>
+      <c r="BN24" s="92"/>
+      <c r="BO24" s="92"/>
+      <c r="BP24" s="52"/>
+      <c r="BQ24" s="53" t="str">
         <f t="shared" si="24"/>
         <v/>
       </c>
-      <c r="Y24" s="58"/>
-      <c r="Z24" s="93"/>
-      <c r="AA24" s="93"/>
-      <c r="AB24" s="52"/>
-      <c r="AC24" s="53" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="AD24" s="58"/>
-      <c r="AE24" s="93"/>
-      <c r="AF24" s="93"/>
-      <c r="AG24" s="52"/>
-      <c r="AH24" s="53" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="AI24" s="58"/>
-      <c r="AJ24" s="93"/>
-      <c r="AK24" s="93"/>
-      <c r="AL24" s="52"/>
-      <c r="AM24" s="53" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="AN24" s="58"/>
-      <c r="AO24" s="93"/>
-      <c r="AP24" s="93"/>
-      <c r="AQ24" s="52"/>
-      <c r="AR24" s="53" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="AS24" s="58"/>
-      <c r="AT24" s="93"/>
-      <c r="AU24" s="93"/>
-      <c r="AV24" s="52"/>
-      <c r="AW24" s="53" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="AX24" s="58"/>
-      <c r="AY24" s="93"/>
-      <c r="AZ24" s="93"/>
-      <c r="BA24" s="52"/>
-      <c r="BB24" s="53" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="BC24" s="58"/>
-      <c r="BD24" s="93"/>
-      <c r="BE24" s="93"/>
-      <c r="BF24" s="52"/>
-      <c r="BG24" s="53" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="BH24" s="58"/>
-      <c r="BI24" s="93"/>
-      <c r="BJ24" s="93"/>
-      <c r="BK24" s="52"/>
-      <c r="BL24" s="53" t="str">
-        <f t="shared" si="21"/>
-        <v/>
-      </c>
-      <c r="BM24" s="58"/>
-      <c r="BN24" s="93"/>
-      <c r="BO24" s="93"/>
-      <c r="BP24" s="52"/>
-      <c r="BQ24" s="53" t="str">
-        <f t="shared" si="22"/>
-        <v/>
-      </c>
       <c r="BR24" s="51">
         <f t="shared" ref="BR24:BR25" si="26">SUM(IF(M24&lt;&gt;"",M24,IF(L24&lt;&gt;"",L24,K24)),IF(R24&lt;&gt;"",R24,IF(Q24&lt;&gt;"",Q24,P24)),IF(W24&lt;&gt;"",W24,IF(V24&lt;&gt;"",V24,U24)),IF(AB24&lt;&gt;"",AB24,IF(AA24&lt;&gt;"",AA24,Z24)),IF(AG24&lt;&gt;"",AG24,IF(AF24&lt;&gt;"",AF24,AE24)),IF(AL24&lt;&gt;"",AL24,IF(AK24&lt;&gt;"",AK24,AJ24)),IF(AQ24&lt;&gt;"",AQ24,IF(AP24&lt;&gt;"",AP24,AO24)),IF(AV24&lt;&gt;"",AV24,IF(AU24&lt;&gt;"",AU24,AT24)),IF(BA24&lt;&gt;"",BA24,IF(AZ24&lt;&gt;"",AZ24,AY24)),IF(BF24&lt;&gt;"",BF24,IF(BE24&lt;&gt;"",BE24,BD24)),IF(BK24&lt;&gt;"",BK24,IF(BJ24&lt;&gt;"",BJ24,BI24)),IF(BP24&lt;&gt;"",BP24,IF(BO24&lt;&gt;"",BO24,BN24)))</f>
         <v>0</v>
       </c>
-      <c r="BS24" s="94"/>
-      <c r="BT24" s="95"/>
+      <c r="BS24" s="93"/>
+      <c r="BT24" s="94"/>
     </row>
     <row r="25" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="59" t="s">
@@ -3633,8 +3638,8 @@
       <c r="B25" s="60" t="s">
         <v>92</v>
       </c>
-      <c r="C25" s="96"/>
-      <c r="D25" s="96"/>
+      <c r="C25" s="95"/>
+      <c r="D25" s="95"/>
       <c r="E25" s="60" t="s">
         <v>92</v>
       </c>
@@ -3649,7 +3654,7 @@
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=1,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),0)</f>
         <v>0</v>
       </c>
-      <c r="N25" s="97" t="str">
+      <c r="N25" s="96" t="str">
         <f t="shared" ca="1" si="25"/>
         <v/>
       </c>
@@ -3745,8 +3750,8 @@
         <f t="shared" ca="1" si="26"/>
         <v>0</v>
       </c>
-      <c r="BS25" s="98"/>
-      <c r="BT25" s="99"/>
+      <c r="BS25" s="97"/>
+      <c r="BT25" s="98"/>
     </row>
     <row r="26" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -3756,6 +3761,29 @@
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="BM11:BQ11"/>
+    <mergeCell ref="BM13:BQ13"/>
+    <mergeCell ref="O11:S11"/>
+    <mergeCell ref="J11:N11"/>
+    <mergeCell ref="T11:X11"/>
+    <mergeCell ref="Y11:AC11"/>
+    <mergeCell ref="AD11:AH11"/>
+    <mergeCell ref="AI11:AM11"/>
+    <mergeCell ref="AN11:AR11"/>
+    <mergeCell ref="AS11:AW11"/>
+    <mergeCell ref="AX11:BB11"/>
+    <mergeCell ref="BC11:BG11"/>
+    <mergeCell ref="BH11:BL11"/>
+    <mergeCell ref="O13:S13"/>
+    <mergeCell ref="J13:N13"/>
+    <mergeCell ref="T13:X13"/>
+    <mergeCell ref="BC12:BG12"/>
+    <mergeCell ref="BH12:BL12"/>
+    <mergeCell ref="Y13:AC13"/>
+    <mergeCell ref="AD13:AH13"/>
+    <mergeCell ref="AI13:AM13"/>
+    <mergeCell ref="AN13:AR13"/>
+    <mergeCell ref="AS13:AW13"/>
     <mergeCell ref="BM12:BQ12"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="H12:I12"/>
@@ -3772,29 +3800,6 @@
     <mergeCell ref="AN12:AR12"/>
     <mergeCell ref="AS12:AW12"/>
     <mergeCell ref="AX12:BB12"/>
-    <mergeCell ref="BC12:BG12"/>
-    <mergeCell ref="BH12:BL12"/>
-    <mergeCell ref="Y13:AC13"/>
-    <mergeCell ref="AD13:AH13"/>
-    <mergeCell ref="AI13:AM13"/>
-    <mergeCell ref="AN13:AR13"/>
-    <mergeCell ref="AS13:AW13"/>
-    <mergeCell ref="BM11:BQ11"/>
-    <mergeCell ref="BM13:BQ13"/>
-    <mergeCell ref="O11:S11"/>
-    <mergeCell ref="J11:N11"/>
-    <mergeCell ref="T11:X11"/>
-    <mergeCell ref="Y11:AC11"/>
-    <mergeCell ref="AD11:AH11"/>
-    <mergeCell ref="AI11:AM11"/>
-    <mergeCell ref="AN11:AR11"/>
-    <mergeCell ref="AS11:AW11"/>
-    <mergeCell ref="AX11:BB11"/>
-    <mergeCell ref="BC11:BG11"/>
-    <mergeCell ref="BH11:BL11"/>
-    <mergeCell ref="O13:S13"/>
-    <mergeCell ref="J13:N13"/>
-    <mergeCell ref="T13:X13"/>
   </mergeCells>
   <conditionalFormatting sqref="M15:M24 R15:R24 W15:W24 AB15:AB24 AG15:AG24 AL15:AL24 AQ15:AQ24 AV15:AV24 BA15:BA24 BF15:BF24 BK15:BK24 BP15:BP24">
     <cfRule type="expression" dxfId="8" priority="8">
@@ -3802,37 +3807,37 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BP10 R15:T24 X15:Y24 AC15:AD24 AH15:AI24 AM15:AN24 AR15:AS24 AW15:AX24 BB15:BC24 BG15:BH24 BL15:BM24 BQ15:BQ24">
-    <cfRule type="expression" dxfId="0" priority="9">
+    <cfRule type="expression" dxfId="1" priority="9">
       <formula>IF(AND(Q10&lt;&gt;"",R10="",TODAY()&gt;DATE(YEAR(TODAY()),MONTH(DATEVALUE("1-"&amp;LEFT(#REF!,3)&amp;"-1900")),20)),TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BR15">
-    <cfRule type="cellIs" dxfId="6" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThan">
       <formula>90%*$G$15</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BR16">
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="greaterThan">
       <formula>90%*$G$16</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BR17">
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
       <formula>90%*$G$17</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BR18">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="greaterThan">
       <formula>90%*$G$18</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BR19">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="greaterThan">
       <formula>90%*$G$19</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BS11:BS12">
-    <cfRule type="expression" dxfId="1" priority="7">
+    <cfRule type="expression" dxfId="2" priority="7">
       <formula>IF(BS11&lt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3843,14 +3848,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19b1ad6d-7bbd-4338-adb0-a51e11e836c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4091,27 +4094,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19b1ad6d-7bbd-4338-adb0-a51e11e836c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BC2B212-31BA-49FB-B215-9E14B2C60948}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="19b1ad6d-7bbd-4338-adb0-a51e11e836c7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4136,9 +4132,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BC2B212-31BA-49FB-B215-9E14B2C60948}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="19b1ad6d-7bbd-4338-adb0-a51e11e836c7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
removed PO box in UI
Removed PO box on UI and replaced with template upload. Now user uploads template w/ filled out POs, pipeline populates sheet.
</commit_message>
<xml_diff>
--- a/data/Financial Spreadsheet Template v2.xlsx
+++ b/data/Financial Spreadsheet Template v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfizer-my.sharepoint.com/personal/hoveyo_pfizer_com/Documents/financial-automation-project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="631" documentId="8_{ADF84F62-CC85-48F6-A2B9-288B99318624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5A7AF0B-2BF2-4B61-9C9A-5B6EDF1F667E}"/>
+  <xr:revisionPtr revIDLastSave="632" documentId="8_{ADF84F62-CC85-48F6-A2B9-288B99318624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6F2359F-4178-4731-A4B9-806048A93478}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="12480" tabRatio="590" xr2:uid="{0996C49B-04E6-42AE-AA83-2F64BE89A626}"/>
   </bookViews>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="100">
   <si>
     <t xml:space="preserve">Overall Capital </t>
   </si>
@@ -405,6 +405,12 @@
   </si>
   <si>
     <t>2/29/2025</t>
+  </si>
+  <si>
+    <t>9500879389</t>
+  </si>
+  <si>
+    <t>9500882917</t>
   </si>
 </sst>
 </file>
@@ -1374,6 +1380,15 @@
     <xf numFmtId="3" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1392,15 +1407,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency 2" xfId="2" xr:uid="{C819F491-96B6-415F-B3EE-ED5A59A1E95E}"/>
@@ -1408,18 +1414,11 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2 2" xfId="3" xr:uid="{EFDA3BDD-7E2C-4F3B-BEB7-091BB23895D4}"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1461,7 +1460,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFFF7C80"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1962,10 +1961,10 @@
         <f ca="1">SUM(J11:X11,Y12:BQ12)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="132" t="s">
+      <c r="H11" s="135" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="133"/>
+      <c r="I11" s="136"/>
       <c r="J11" s="129" cm="1">
         <f t="array" aca="1" ref="J11" ca="1">SUM(M15:M25)+SUM(_xlfn._xlws.FILTER(L15:L25,M15:M25=""))+SUM(_xlfn._xlws.FILTER(K15:K25,(L15:L25="")*(M15:M25="")))+SUMIFS(N15:N25,M15:M25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(J15:J25)</f>
         <v>0</v>
@@ -2093,10 +2092,10 @@
         <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="134" t="s">
+      <c r="H12" s="137" t="s">
         <v>16</v>
       </c>
-      <c r="I12" s="135"/>
+      <c r="I12" s="138"/>
       <c r="J12" s="129" cm="1">
         <f t="array" aca="1" ref="J12" ca="1">SUM(M15:M25)+SUM(_xlfn._xlws.FILTER(L15:L25,M15:M25=""))+SUM(_xlfn._xlws.FILTER(K15:K25,(L15:L25="")*(M15:M25="")))</f>
         <v>0</v>
@@ -2200,116 +2199,116 @@
       <c r="A13" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="136" t="s">
+      <c r="H13" s="139" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="137"/>
-      <c r="J13" s="138">
+      <c r="I13" s="140"/>
+      <c r="J13" s="132">
         <v>45688</v>
       </c>
-      <c r="K13" s="139" t="s">
+      <c r="K13" s="133" t="s">
         <v>19</v>
       </c>
-      <c r="L13" s="139"/>
-      <c r="M13" s="139"/>
-      <c r="N13" s="139"/>
-      <c r="O13" s="138" t="s">
+      <c r="L13" s="133"/>
+      <c r="M13" s="133"/>
+      <c r="N13" s="133"/>
+      <c r="O13" s="132" t="s">
         <v>97</v>
       </c>
-      <c r="P13" s="139"/>
-      <c r="Q13" s="139"/>
-      <c r="R13" s="139"/>
-      <c r="S13" s="140"/>
-      <c r="T13" s="138">
+      <c r="P13" s="133"/>
+      <c r="Q13" s="133"/>
+      <c r="R13" s="133"/>
+      <c r="S13" s="134"/>
+      <c r="T13" s="132">
         <v>45747</v>
       </c>
-      <c r="U13" s="139" t="s">
+      <c r="U13" s="133" t="s">
         <v>20</v>
       </c>
-      <c r="V13" s="139"/>
-      <c r="W13" s="139"/>
-      <c r="X13" s="140"/>
-      <c r="Y13" s="138">
+      <c r="V13" s="133"/>
+      <c r="W13" s="133"/>
+      <c r="X13" s="134"/>
+      <c r="Y13" s="132">
         <v>45777</v>
       </c>
-      <c r="Z13" s="139" t="s">
+      <c r="Z13" s="133" t="s">
         <v>21</v>
       </c>
-      <c r="AA13" s="139"/>
-      <c r="AB13" s="139"/>
-      <c r="AC13" s="140"/>
-      <c r="AD13" s="138">
+      <c r="AA13" s="133"/>
+      <c r="AB13" s="133"/>
+      <c r="AC13" s="134"/>
+      <c r="AD13" s="132">
         <v>45808</v>
       </c>
-      <c r="AE13" s="139" t="s">
+      <c r="AE13" s="133" t="s">
         <v>22</v>
       </c>
-      <c r="AF13" s="139"/>
-      <c r="AG13" s="139"/>
-      <c r="AH13" s="140"/>
-      <c r="AI13" s="138">
+      <c r="AF13" s="133"/>
+      <c r="AG13" s="133"/>
+      <c r="AH13" s="134"/>
+      <c r="AI13" s="132">
         <v>45838</v>
       </c>
-      <c r="AJ13" s="139" t="s">
+      <c r="AJ13" s="133" t="s">
         <v>23</v>
       </c>
-      <c r="AK13" s="139"/>
-      <c r="AL13" s="139"/>
-      <c r="AM13" s="140"/>
-      <c r="AN13" s="138">
+      <c r="AK13" s="133"/>
+      <c r="AL13" s="133"/>
+      <c r="AM13" s="134"/>
+      <c r="AN13" s="132">
         <v>45869</v>
       </c>
-      <c r="AO13" s="139" t="s">
+      <c r="AO13" s="133" t="s">
         <v>24</v>
       </c>
-      <c r="AP13" s="139"/>
-      <c r="AQ13" s="139"/>
-      <c r="AR13" s="140"/>
-      <c r="AS13" s="138">
+      <c r="AP13" s="133"/>
+      <c r="AQ13" s="133"/>
+      <c r="AR13" s="134"/>
+      <c r="AS13" s="132">
         <v>45900</v>
       </c>
-      <c r="AT13" s="139" t="s">
+      <c r="AT13" s="133" t="s">
         <v>25</v>
       </c>
-      <c r="AU13" s="139"/>
-      <c r="AV13" s="139"/>
-      <c r="AW13" s="140"/>
-      <c r="AX13" s="138">
+      <c r="AU13" s="133"/>
+      <c r="AV13" s="133"/>
+      <c r="AW13" s="134"/>
+      <c r="AX13" s="132">
         <v>45930</v>
       </c>
-      <c r="AY13" s="139" t="s">
+      <c r="AY13" s="133" t="s">
         <v>26</v>
       </c>
-      <c r="AZ13" s="139"/>
-      <c r="BA13" s="139"/>
-      <c r="BB13" s="140"/>
-      <c r="BC13" s="138">
+      <c r="AZ13" s="133"/>
+      <c r="BA13" s="133"/>
+      <c r="BB13" s="134"/>
+      <c r="BC13" s="132">
         <v>45961</v>
       </c>
-      <c r="BD13" s="139" t="s">
+      <c r="BD13" s="133" t="s">
         <v>27</v>
       </c>
-      <c r="BE13" s="139"/>
-      <c r="BF13" s="139"/>
-      <c r="BG13" s="140"/>
-      <c r="BH13" s="138">
+      <c r="BE13" s="133"/>
+      <c r="BF13" s="133"/>
+      <c r="BG13" s="134"/>
+      <c r="BH13" s="132">
         <v>45991</v>
       </c>
-      <c r="BI13" s="139" t="s">
+      <c r="BI13" s="133" t="s">
         <v>28</v>
       </c>
-      <c r="BJ13" s="139"/>
-      <c r="BK13" s="139"/>
-      <c r="BL13" s="140"/>
-      <c r="BM13" s="138">
+      <c r="BJ13" s="133"/>
+      <c r="BK13" s="133"/>
+      <c r="BL13" s="134"/>
+      <c r="BM13" s="132">
         <v>46022</v>
       </c>
-      <c r="BN13" s="139" t="s">
+      <c r="BN13" s="133" t="s">
         <v>29</v>
       </c>
-      <c r="BO13" s="139"/>
-      <c r="BP13" s="139"/>
-      <c r="BQ13" s="140"/>
+      <c r="BO13" s="133"/>
+      <c r="BP13" s="133"/>
+      <c r="BQ13" s="134"/>
       <c r="BR13" s="24">
         <f>SUM(BR15:BR24)</f>
         <v>0</v>
@@ -2537,7 +2536,9 @@
     </row>
     <row r="15" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A15" s="39"/>
-      <c r="B15" s="40"/>
+      <c r="B15" s="40" t="s">
+        <v>98</v>
+      </c>
       <c r="C15" s="69"/>
       <c r="D15" s="69"/>
       <c r="E15" s="40"/>
@@ -2650,7 +2651,9 @@
     </row>
     <row r="16" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A16" s="47"/>
-      <c r="B16" s="48"/>
+      <c r="B16" s="48" t="s">
+        <v>99</v>
+      </c>
       <c r="C16" s="72"/>
       <c r="D16" s="72"/>
       <c r="E16" s="72"/>
@@ -3761,6 +3764,29 @@
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="BM12:BQ12"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="AX13:BB13"/>
+    <mergeCell ref="BC13:BG13"/>
+    <mergeCell ref="BH13:BL13"/>
+    <mergeCell ref="J12:N12"/>
+    <mergeCell ref="O12:S12"/>
+    <mergeCell ref="T12:X12"/>
+    <mergeCell ref="Y12:AC12"/>
+    <mergeCell ref="AD12:AH12"/>
+    <mergeCell ref="AI12:AM12"/>
+    <mergeCell ref="AN12:AR12"/>
+    <mergeCell ref="AS12:AW12"/>
+    <mergeCell ref="AX12:BB12"/>
+    <mergeCell ref="BC12:BG12"/>
+    <mergeCell ref="BH12:BL12"/>
+    <mergeCell ref="Y13:AC13"/>
+    <mergeCell ref="AD13:AH13"/>
+    <mergeCell ref="AI13:AM13"/>
+    <mergeCell ref="AN13:AR13"/>
+    <mergeCell ref="AS13:AW13"/>
     <mergeCell ref="BM11:BQ11"/>
     <mergeCell ref="BM13:BQ13"/>
     <mergeCell ref="O11:S11"/>
@@ -3777,67 +3803,44 @@
     <mergeCell ref="O13:S13"/>
     <mergeCell ref="J13:N13"/>
     <mergeCell ref="T13:X13"/>
-    <mergeCell ref="BC12:BG12"/>
-    <mergeCell ref="BH12:BL12"/>
-    <mergeCell ref="Y13:AC13"/>
-    <mergeCell ref="AD13:AH13"/>
-    <mergeCell ref="AI13:AM13"/>
-    <mergeCell ref="AN13:AR13"/>
-    <mergeCell ref="AS13:AW13"/>
-    <mergeCell ref="BM12:BQ12"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="AX13:BB13"/>
-    <mergeCell ref="BC13:BG13"/>
-    <mergeCell ref="BH13:BL13"/>
-    <mergeCell ref="J12:N12"/>
-    <mergeCell ref="O12:S12"/>
-    <mergeCell ref="T12:X12"/>
-    <mergeCell ref="Y12:AC12"/>
-    <mergeCell ref="AD12:AH12"/>
-    <mergeCell ref="AI12:AM12"/>
-    <mergeCell ref="AN12:AR12"/>
-    <mergeCell ref="AS12:AW12"/>
-    <mergeCell ref="AX12:BB12"/>
   </mergeCells>
   <conditionalFormatting sqref="M15:M24 R15:R24 W15:W24 AB15:AB24 AG15:AG24 AL15:AL24 AQ15:AQ24 AV15:AV24 BA15:BA24 BF15:BF24 BK15:BK24 BP15:BP24">
-    <cfRule type="expression" dxfId="8" priority="8">
+    <cfRule type="expression" dxfId="7" priority="8">
       <formula>IF(AND(L15&gt;0,M15=0),TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BP10 R15:T24 X15:Y24 AC15:AD24 AH15:AI24 AM15:AN24 AR15:AS24 AW15:AX24 BB15:BC24 BG15:BH24 BL15:BM24 BQ15:BQ24">
-    <cfRule type="expression" dxfId="1" priority="9">
+    <cfRule type="expression" dxfId="6" priority="9">
       <formula>IF(AND(Q10&lt;&gt;"",R10="",TODAY()&gt;DATE(YEAR(TODAY()),MONTH(DATEVALUE("1-"&amp;LEFT(#REF!,3)&amp;"-1900")),20)),TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BR15">
-    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
       <formula>90%*$G$15</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BR16">
-    <cfRule type="cellIs" dxfId="6" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="greaterThan">
       <formula>90%*$G$16</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BR17">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
       <formula>90%*$G$17</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BR18">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
       <formula>90%*$G$18</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BR19">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
       <formula>90%*$G$19</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BS11:BS12">
-    <cfRule type="expression" dxfId="2" priority="7">
+    <cfRule type="expression" dxfId="0" priority="7">
       <formula>IF(BS11&lt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3848,12 +3851,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19b1ad6d-7bbd-4338-adb0-a51e11e836c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4094,20 +4099,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19b1ad6d-7bbd-4338-adb0-a51e11e836c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BC2B212-31BA-49FB-B215-9E14B2C60948}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="19b1ad6d-7bbd-4338-adb0-a51e11e836c7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4132,18 +4144,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BC2B212-31BA-49FB-B215-9E14B2C60948}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="19b1ad6d-7bbd-4338-adb0-a51e11e836c7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update test notebook (minor)
</commit_message>
<xml_diff>
--- a/data/Financial Spreadsheet Template v2.xlsx
+++ b/data/Financial Spreadsheet Template v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfizer-my.sharepoint.com/personal/hoveyo_pfizer_com/Documents/financial-automation-project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="632" documentId="8_{ADF84F62-CC85-48F6-A2B9-288B99318624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6F2359F-4178-4731-A4B9-806048A93478}"/>
+  <xr:revisionPtr revIDLastSave="638" documentId="8_{ADF84F62-CC85-48F6-A2B9-288B99318624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C4F8E26-0597-41F5-8C7D-1D569EEE31E4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="12480" tabRatio="590" xr2:uid="{0996C49B-04E6-42AE-AA83-2F64BE89A626}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="14250" tabRatio="590" xr2:uid="{0996C49B-04E6-42AE-AA83-2F64BE89A626}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="5" r:id="rId1"/>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="107">
   <si>
     <t xml:space="preserve">Overall Capital </t>
   </si>
@@ -412,18 +412,40 @@
   <si>
     <t>9500882917</t>
   </si>
+  <si>
+    <t>IT PO</t>
+  </si>
+  <si>
+    <t>IBM</t>
+  </si>
+  <si>
+    <t>IT-FBT0790-OG-US-00</t>
+  </si>
+  <si>
+    <t>IO Support - IBM 2025 S1 - IO support-GARITD IBM 2025 S1 - IO support[42]</t>
+  </si>
+  <si>
+    <t>OPEN</t>
+  </si>
+  <si>
+    <t>IT-FBT0545-OG-US-00</t>
+  </si>
+  <si>
+    <t>Covid Support - IBM - 2025 S1 Covid applications support</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="[$-409]dd\-mmm\-yy;@"/>
     <numFmt numFmtId="166" formatCode="mmmm\-yyyy"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -521,6 +543,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1191,7 +1220,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="149">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1263,10 +1292,8 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="23" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1295,7 +1322,6 @@
     <xf numFmtId="164" fontId="9" fillId="2" borderId="45" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1380,15 +1406,6 @@
     <xf numFmtId="3" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1407,6 +1424,30 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="13" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency 2" xfId="2" xr:uid="{C819F491-96B6-415F-B3EE-ED5A59A1E95E}"/>
@@ -1836,7 +1877,7 @@
       <c r="E3" s="7">
         <v>2025</v>
       </c>
-      <c r="F3" s="127">
+      <c r="F3" s="124">
         <f>C3</f>
         <v>0</v>
       </c>
@@ -1860,7 +1901,7 @@
       <c r="E4" s="7">
         <v>2025</v>
       </c>
-      <c r="F4" s="127">
+      <c r="F4" s="124">
         <v>0</v>
       </c>
     </row>
@@ -1872,7 +1913,7 @@
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
-      <c r="F5" s="128"/>
+      <c r="F5" s="125"/>
     </row>
     <row r="6" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
@@ -1883,7 +1924,7 @@
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
-      <c r="E6" s="112" t="str">
+      <c r="E6" s="109" t="str">
         <f ca="1">IF(SUMIFS(BR:BR,A:A,"Contingency")&gt;0,"Contingency is "&amp;TEXT(SUMIFS(BR:BR,A:A,"Contingency"),"$#,##"),IF(SUMIFS(BR:BR,A:A,"Contingency")&lt;0,"Overspent by "&amp;TEXT(SUMIFS(BR:BR,A:A,"Contingency"),"$#,##"),"No contingency"))</f>
         <v>No contingency</v>
       </c>
@@ -1891,9 +1932,9 @@
     </row>
     <row r="7" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A7" s="13"/>
-      <c r="B7" s="111"/>
-      <c r="C7" s="110"/>
-      <c r="D7" s="110"/>
+      <c r="B7" s="108"/>
+      <c r="C7" s="107"/>
+      <c r="D7" s="107"/>
       <c r="E7" s="14"/>
       <c r="F7" s="15"/>
       <c r="O7" s="16"/>
@@ -1909,158 +1950,158 @@
         <f>C4-BR13</f>
         <v>0</v>
       </c>
-      <c r="D9" s="113"/>
-      <c r="E9" s="119" t="s">
+      <c r="D9" s="110"/>
+      <c r="E9" s="116" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="119" t="s">
+      <c r="F9" s="116" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="120" t="s">
+      <c r="G9" s="117" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="125" t="s">
+      <c r="A10" s="122" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="126" t="e">
+      <c r="B10" s="123" t="e">
         <f>B9/C4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D10" s="121" t="s">
+      <c r="D10" s="118" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="114"/>
-      <c r="F10" s="114"/>
-      <c r="G10" s="115"/>
-      <c r="BS10" s="67" t="s">
+      <c r="E10" s="111"/>
+      <c r="F10" s="111"/>
+      <c r="G10" s="112"/>
+      <c r="BS10" s="65" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:73" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="123" t="s">
+      <c r="A11" s="120" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="124">
+      <c r="B11" s="121">
         <f ca="1">SUMIFS(J12:BQ12,J13:BQ13,"&lt;="&amp;TODAY())</f>
         <v>0</v>
       </c>
-      <c r="D11" s="121" t="s">
+      <c r="D11" s="118" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="114">
+      <c r="E11" s="111">
         <f ca="1">SUM(J11:X11,Y12:AM12)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="114">
+      <c r="F11" s="111">
         <f ca="1">SUM(AN12:BQ12)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="115">
+      <c r="G11" s="112">
         <f ca="1">SUM(J11:X11,Y12:BQ12)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="135" t="s">
+      <c r="H11" s="129" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="136"/>
-      <c r="J11" s="129" cm="1">
+      <c r="I11" s="130"/>
+      <c r="J11" s="126" cm="1">
         <f t="array" aca="1" ref="J11" ca="1">SUM(M15:M25)+SUM(_xlfn._xlws.FILTER(L15:L25,M15:M25=""))+SUM(_xlfn._xlws.FILTER(K15:K25,(L15:L25="")*(M15:M25="")))+SUMIFS(N15:N25,M15:M25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(J15:J25)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="130"/>
-      <c r="L11" s="130"/>
-      <c r="M11" s="130"/>
-      <c r="N11" s="131"/>
-      <c r="O11" s="129" cm="1">
+      <c r="K11" s="127"/>
+      <c r="L11" s="127"/>
+      <c r="M11" s="127"/>
+      <c r="N11" s="128"/>
+      <c r="O11" s="126" cm="1">
         <f t="array" aca="1" ref="O11" ca="1">SUM(R15:R25)+SUM(_xlfn._xlws.FILTER(Q15:Q25,R15:R25=""))+SUM(_xlfn._xlws.FILTER(P15:P25,(Q15:Q25="")*(R15:R25="")))+SUMIFS(S15:S25,R15:R25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(O15:O25)</f>
         <v>0</v>
       </c>
-      <c r="P11" s="130"/>
-      <c r="Q11" s="130"/>
-      <c r="R11" s="130"/>
-      <c r="S11" s="131"/>
-      <c r="T11" s="129" cm="1">
+      <c r="P11" s="127"/>
+      <c r="Q11" s="127"/>
+      <c r="R11" s="127"/>
+      <c r="S11" s="128"/>
+      <c r="T11" s="126" cm="1">
         <f t="array" aca="1" ref="T11" ca="1">SUM(W15:W25)+SUM(_xlfn._xlws.FILTER(V15:V25,W15:W25=""))+SUM(_xlfn._xlws.FILTER(U15:U25,(V15:V25="")*(W15:W25="")))+SUMIFS(X15:X25,W15:W25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(T15:T25)</f>
         <v>0</v>
       </c>
-      <c r="U11" s="130"/>
-      <c r="V11" s="130"/>
-      <c r="W11" s="130"/>
-      <c r="X11" s="131"/>
-      <c r="Y11" s="129" cm="1">
+      <c r="U11" s="127"/>
+      <c r="V11" s="127"/>
+      <c r="W11" s="127"/>
+      <c r="X11" s="128"/>
+      <c r="Y11" s="126" cm="1">
         <f t="array" aca="1" ref="Y11" ca="1">SUM(AB15:AB25)+SUM(_xlfn._xlws.FILTER(AA15:AA25,AB15:AB25=""))+SUM(_xlfn._xlws.FILTER(Z15:Z25,(AA15:AA25="")*(AB15:AB25="")))+SUMIFS(AC15:AC25,AB15:AB25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(Y15:Y25)</f>
         <v>0</v>
       </c>
-      <c r="Z11" s="130"/>
-      <c r="AA11" s="130"/>
-      <c r="AB11" s="130"/>
-      <c r="AC11" s="131"/>
-      <c r="AD11" s="129" cm="1">
+      <c r="Z11" s="127"/>
+      <c r="AA11" s="127"/>
+      <c r="AB11" s="127"/>
+      <c r="AC11" s="128"/>
+      <c r="AD11" s="126" cm="1">
         <f t="array" aca="1" ref="AD11" ca="1">SUM(AG15:AG25)+SUM(_xlfn._xlws.FILTER(AF15:AF25,AG15:AG25=""))+SUM(_xlfn._xlws.FILTER(AE15:AE25,(AF15:AF25="")*(AG15:AG25="")))+SUMIFS(AH15:AH25,AG15:AG25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AD15:AD25)</f>
         <v>0</v>
       </c>
-      <c r="AE11" s="130"/>
-      <c r="AF11" s="130"/>
-      <c r="AG11" s="130"/>
-      <c r="AH11" s="131"/>
-      <c r="AI11" s="129" cm="1">
+      <c r="AE11" s="127"/>
+      <c r="AF11" s="127"/>
+      <c r="AG11" s="127"/>
+      <c r="AH11" s="128"/>
+      <c r="AI11" s="126" cm="1">
         <f t="array" aca="1" ref="AI11" ca="1">SUM(AL15:AL25)+SUM(_xlfn._xlws.FILTER(AK15:AK25,AL15:AL25=""))+SUM(_xlfn._xlws.FILTER(AJ15:AJ25,(AK15:AK25="")*(AL15:AL25="")))+SUMIFS(AM15:AM25,AL15:AL25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AI15:AI25)</f>
         <v>0</v>
       </c>
-      <c r="AJ11" s="130"/>
-      <c r="AK11" s="130"/>
-      <c r="AL11" s="130"/>
-      <c r="AM11" s="131"/>
-      <c r="AN11" s="129" cm="1">
+      <c r="AJ11" s="127"/>
+      <c r="AK11" s="127"/>
+      <c r="AL11" s="127"/>
+      <c r="AM11" s="128"/>
+      <c r="AN11" s="126" cm="1">
         <f t="array" aca="1" ref="AN11" ca="1">SUM(AQ15:AQ25)+SUM(_xlfn._xlws.FILTER(AP15:AP25,AQ15:AQ25=""))+SUM(_xlfn._xlws.FILTER(AO15:AO25,(AP15:AP25="")*(AQ15:AQ25="")))+SUMIFS(AR15:AR25,AQ15:AQ25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AN15:AN25)</f>
         <v>0</v>
       </c>
-      <c r="AO11" s="130"/>
-      <c r="AP11" s="130"/>
-      <c r="AQ11" s="130"/>
-      <c r="AR11" s="131"/>
-      <c r="AS11" s="129" cm="1">
+      <c r="AO11" s="127"/>
+      <c r="AP11" s="127"/>
+      <c r="AQ11" s="127"/>
+      <c r="AR11" s="128"/>
+      <c r="AS11" s="126" cm="1">
         <f t="array" aca="1" ref="AS11" ca="1">SUM(AV15:AV25)+SUM(_xlfn._xlws.FILTER(AU15:AU25,AV15:AV25=""))+SUM(_xlfn._xlws.FILTER(AT15:AT25,(AU15:AU25="")*(AV15:AV25="")))+SUMIFS(AW15:AW25,AV15:AV25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AS15:AS25)</f>
         <v>0</v>
       </c>
-      <c r="AT11" s="130"/>
-      <c r="AU11" s="130"/>
-      <c r="AV11" s="130"/>
-      <c r="AW11" s="131"/>
-      <c r="AX11" s="129" cm="1">
+      <c r="AT11" s="127"/>
+      <c r="AU11" s="127"/>
+      <c r="AV11" s="127"/>
+      <c r="AW11" s="128"/>
+      <c r="AX11" s="126" cm="1">
         <f t="array" aca="1" ref="AX11" ca="1">SUM(BA15:BA25)+SUM(_xlfn._xlws.FILTER(AZ15:AZ25,BA15:BA25=""))+SUM(_xlfn._xlws.FILTER(AY15:AY25,(AZ15:AZ25="")*(BA15:BA25="")))+SUMIFS(BB15:BB25,BA15:BA25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AX15:AX25)</f>
         <v>0</v>
       </c>
-      <c r="AY11" s="130"/>
-      <c r="AZ11" s="130"/>
-      <c r="BA11" s="130"/>
-      <c r="BB11" s="131"/>
-      <c r="BC11" s="129" cm="1">
+      <c r="AY11" s="127"/>
+      <c r="AZ11" s="127"/>
+      <c r="BA11" s="127"/>
+      <c r="BB11" s="128"/>
+      <c r="BC11" s="126" cm="1">
         <f t="array" aca="1" ref="BC11" ca="1">SUM(BF15:BF25)+SUM(_xlfn._xlws.FILTER(BE15:BE25,BF15:BF25=""))+SUM(_xlfn._xlws.FILTER(BD15:BD25,(BE15:BE25="")*(BF15:BF25="")))+SUMIFS(BG15:BG25,BF15:BF25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(BC15:BC25)</f>
         <v>0</v>
       </c>
-      <c r="BD11" s="130"/>
-      <c r="BE11" s="130"/>
-      <c r="BF11" s="130"/>
-      <c r="BG11" s="131"/>
-      <c r="BH11" s="129" cm="1">
+      <c r="BD11" s="127"/>
+      <c r="BE11" s="127"/>
+      <c r="BF11" s="127"/>
+      <c r="BG11" s="128"/>
+      <c r="BH11" s="126" cm="1">
         <f t="array" aca="1" ref="BH11" ca="1">SUM(BK15:BK25)+SUM(_xlfn._xlws.FILTER(BJ15:BJ25,BK15:BK25=""))+SUM(_xlfn._xlws.FILTER(BI15:BI25,(BJ15:BJ25="")*(BK15:BK25="")))+SUMIFS(BL15:BL25,BK15:BK25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(BH15:BH25)</f>
         <v>0</v>
       </c>
-      <c r="BI11" s="130"/>
-      <c r="BJ11" s="130"/>
-      <c r="BK11" s="130"/>
-      <c r="BL11" s="131"/>
-      <c r="BM11" s="129" cm="1">
+      <c r="BI11" s="127"/>
+      <c r="BJ11" s="127"/>
+      <c r="BK11" s="127"/>
+      <c r="BL11" s="128"/>
+      <c r="BM11" s="126" cm="1">
         <f t="array" aca="1" ref="BM11" ca="1">SUM(BP15:BP25)+SUM(_xlfn._xlws.FILTER(BO15:BO25,BP15:BP25=""))+SUM(_xlfn._xlws.FILTER(BN15:BN25,(BO15:BO25="")*(BP15:BP25="")))+SUMIFS(BQ15:BQ25,BP15:BP25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(BM15:BM25)</f>
         <v>0</v>
       </c>
-      <c r="BN11" s="130"/>
-      <c r="BO11" s="130"/>
-      <c r="BP11" s="130"/>
-      <c r="BQ11" s="131"/>
+      <c r="BN11" s="127"/>
+      <c r="BO11" s="127"/>
+      <c r="BP11" s="127"/>
+      <c r="BQ11" s="128"/>
       <c r="BR11" s="21" t="s">
         <v>13</v>
       </c>
@@ -2073,125 +2114,125 @@
       <c r="A12" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="118">
+      <c r="B12" s="115">
         <f ca="1">C4-B11</f>
         <v>0</v>
       </c>
-      <c r="D12" s="122" t="s">
+      <c r="D12" s="119" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="116">
+      <c r="E12" s="113">
         <f ca="1">E11-E10</f>
         <v>0</v>
       </c>
-      <c r="F12" s="116">
+      <c r="F12" s="113">
         <f t="shared" ref="F12:G12" ca="1" si="0">F11-F10</f>
         <v>0</v>
       </c>
-      <c r="G12" s="117">
+      <c r="G12" s="114">
         <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="137" t="s">
+      <c r="H12" s="131" t="s">
         <v>16</v>
       </c>
-      <c r="I12" s="138"/>
-      <c r="J12" s="129" cm="1">
+      <c r="I12" s="132"/>
+      <c r="J12" s="126" cm="1">
         <f t="array" aca="1" ref="J12" ca="1">SUM(M15:M25)+SUM(_xlfn._xlws.FILTER(L15:L25,M15:M25=""))+SUM(_xlfn._xlws.FILTER(K15:K25,(L15:L25="")*(M15:M25="")))</f>
         <v>0</v>
       </c>
-      <c r="K12" s="130"/>
-      <c r="L12" s="130"/>
-      <c r="M12" s="130"/>
-      <c r="N12" s="131"/>
-      <c r="O12" s="129" cm="1">
+      <c r="K12" s="127"/>
+      <c r="L12" s="127"/>
+      <c r="M12" s="127"/>
+      <c r="N12" s="128"/>
+      <c r="O12" s="126" cm="1">
         <f t="array" aca="1" ref="O12" ca="1">SUM(R15:R25)+SUM(_xlfn._xlws.FILTER(Q15:Q25,R15:R25=""))+SUM(_xlfn._xlws.FILTER(P15:P25,(Q15:Q25="")*(R15:R25="")))</f>
         <v>0</v>
       </c>
-      <c r="P12" s="130"/>
-      <c r="Q12" s="130"/>
-      <c r="R12" s="130"/>
-      <c r="S12" s="131"/>
-      <c r="T12" s="129" cm="1">
+      <c r="P12" s="127"/>
+      <c r="Q12" s="127"/>
+      <c r="R12" s="127"/>
+      <c r="S12" s="128"/>
+      <c r="T12" s="126" cm="1">
         <f t="array" aca="1" ref="T12" ca="1">SUM(W15:W25)+SUM(_xlfn._xlws.FILTER(V15:V25,W15:W25=""))+SUM(_xlfn._xlws.FILTER(U15:U25,(V15:V25="")*(W15:W25="")))</f>
         <v>0</v>
       </c>
-      <c r="U12" s="130"/>
-      <c r="V12" s="130"/>
-      <c r="W12" s="130"/>
-      <c r="X12" s="131"/>
-      <c r="Y12" s="129" cm="1">
+      <c r="U12" s="127"/>
+      <c r="V12" s="127"/>
+      <c r="W12" s="127"/>
+      <c r="X12" s="128"/>
+      <c r="Y12" s="126" cm="1">
         <f t="array" aca="1" ref="Y12" ca="1">SUM(AB15:AB25)+SUM(_xlfn._xlws.FILTER(AA15:AA25,AB15:AB25=""))+SUM(_xlfn._xlws.FILTER(Z15:Z25,(AA15:AA25="")*(AB15:AB25="")))</f>
         <v>0</v>
       </c>
-      <c r="Z12" s="130"/>
-      <c r="AA12" s="130"/>
-      <c r="AB12" s="130"/>
-      <c r="AC12" s="131"/>
-      <c r="AD12" s="129" cm="1">
+      <c r="Z12" s="127"/>
+      <c r="AA12" s="127"/>
+      <c r="AB12" s="127"/>
+      <c r="AC12" s="128"/>
+      <c r="AD12" s="126" cm="1">
         <f t="array" aca="1" ref="AD12" ca="1">SUM(AG15:AG25)+SUM(_xlfn._xlws.FILTER(AF15:AF25,AG15:AG25=""))+SUM(_xlfn._xlws.FILTER(AE15:AE25,(AF15:AF25="")*(AG15:AG25="")))</f>
         <v>0</v>
       </c>
-      <c r="AE12" s="130"/>
-      <c r="AF12" s="130"/>
-      <c r="AG12" s="130"/>
-      <c r="AH12" s="131"/>
-      <c r="AI12" s="129" cm="1">
+      <c r="AE12" s="127"/>
+      <c r="AF12" s="127"/>
+      <c r="AG12" s="127"/>
+      <c r="AH12" s="128"/>
+      <c r="AI12" s="126" cm="1">
         <f t="array" aca="1" ref="AI12" ca="1">SUM(AL15:AL25)+SUM(_xlfn._xlws.FILTER(AK15:AK25,AL15:AL25=""))+SUM(_xlfn._xlws.FILTER(AJ15:AJ25,(AK15:AK25="")*(AL15:AL25="")))</f>
         <v>0</v>
       </c>
-      <c r="AJ12" s="130"/>
-      <c r="AK12" s="130"/>
-      <c r="AL12" s="130"/>
-      <c r="AM12" s="131"/>
-      <c r="AN12" s="129" cm="1">
+      <c r="AJ12" s="127"/>
+      <c r="AK12" s="127"/>
+      <c r="AL12" s="127"/>
+      <c r="AM12" s="128"/>
+      <c r="AN12" s="126" cm="1">
         <f t="array" aca="1" ref="AN12" ca="1">SUM(AQ15:AQ25)+SUM(_xlfn._xlws.FILTER(AP15:AP25,AQ15:AQ25=""))+SUM(_xlfn._xlws.FILTER(AO15:AO25,(AP15:AP25="")*(AQ15:AQ25="")))</f>
         <v>0</v>
       </c>
-      <c r="AO12" s="130"/>
-      <c r="AP12" s="130"/>
-      <c r="AQ12" s="130"/>
-      <c r="AR12" s="131"/>
-      <c r="AS12" s="129" cm="1">
+      <c r="AO12" s="127"/>
+      <c r="AP12" s="127"/>
+      <c r="AQ12" s="127"/>
+      <c r="AR12" s="128"/>
+      <c r="AS12" s="126" cm="1">
         <f t="array" aca="1" ref="AS12" ca="1">SUM(AV15:AV25)+SUM(_xlfn._xlws.FILTER(AU15:AU25,AV15:AV25=""))+SUM(_xlfn._xlws.FILTER(AT15:AT25,(AU15:AU25="")*(AV15:AV25="")))</f>
         <v>0</v>
       </c>
-      <c r="AT12" s="130"/>
-      <c r="AU12" s="130"/>
-      <c r="AV12" s="130"/>
-      <c r="AW12" s="131"/>
-      <c r="AX12" s="129" cm="1">
+      <c r="AT12" s="127"/>
+      <c r="AU12" s="127"/>
+      <c r="AV12" s="127"/>
+      <c r="AW12" s="128"/>
+      <c r="AX12" s="126" cm="1">
         <f t="array" aca="1" ref="AX12" ca="1">SUM(BA15:BA25)+SUM(_xlfn._xlws.FILTER(AZ15:AZ25,BA15:BA25=""))+SUM(_xlfn._xlws.FILTER(AY15:AY25,(AZ15:AZ25="")*(BA15:BA25="")))</f>
         <v>0</v>
       </c>
-      <c r="AY12" s="130"/>
-      <c r="AZ12" s="130"/>
-      <c r="BA12" s="130"/>
-      <c r="BB12" s="131"/>
-      <c r="BC12" s="129" cm="1">
+      <c r="AY12" s="127"/>
+      <c r="AZ12" s="127"/>
+      <c r="BA12" s="127"/>
+      <c r="BB12" s="128"/>
+      <c r="BC12" s="126" cm="1">
         <f t="array" aca="1" ref="BC12" ca="1">SUM(BF15:BF25)+SUM(_xlfn._xlws.FILTER(BE15:BE25,BF15:BF25=""))+SUM(_xlfn._xlws.FILTER(BD15:BD25,(BE15:BE25="")*(BF15:BF25="")))</f>
         <v>0</v>
       </c>
-      <c r="BD12" s="130"/>
-      <c r="BE12" s="130"/>
-      <c r="BF12" s="130"/>
-      <c r="BG12" s="131"/>
-      <c r="BH12" s="129" cm="1">
+      <c r="BD12" s="127"/>
+      <c r="BE12" s="127"/>
+      <c r="BF12" s="127"/>
+      <c r="BG12" s="128"/>
+      <c r="BH12" s="126" cm="1">
         <f t="array" aca="1" ref="BH12" ca="1">SUM(BK15:BK25)+SUM(_xlfn._xlws.FILTER(BJ15:BJ25,BK15:BK25=""))+SUM(_xlfn._xlws.FILTER(BI15:BI25,(BJ15:BJ25="")*(BK15:BK25="")))</f>
         <v>0</v>
       </c>
-      <c r="BI12" s="130"/>
-      <c r="BJ12" s="130"/>
-      <c r="BK12" s="130"/>
-      <c r="BL12" s="131"/>
-      <c r="BM12" s="129" cm="1">
+      <c r="BI12" s="127"/>
+      <c r="BJ12" s="127"/>
+      <c r="BK12" s="127"/>
+      <c r="BL12" s="128"/>
+      <c r="BM12" s="126" cm="1">
         <f t="array" aca="1" ref="BM12" ca="1">SUM(BP15:BP25)+SUM(_xlfn._xlws.FILTER(BO15:BO25,BP15:BP25=""))+SUM(_xlfn._xlws.FILTER(BN15:BN25,(BO15:BO25="")*(BP15:BP25="")))</f>
         <v>0</v>
       </c>
-      <c r="BN12" s="130"/>
-      <c r="BO12" s="130"/>
-      <c r="BP12" s="130"/>
-      <c r="BQ12" s="131"/>
+      <c r="BN12" s="127"/>
+      <c r="BO12" s="127"/>
+      <c r="BP12" s="127"/>
+      <c r="BQ12" s="128"/>
       <c r="BR12" s="21"/>
       <c r="BS12" s="22"/>
     </row>
@@ -2199,116 +2240,116 @@
       <c r="A13" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="139" t="s">
+      <c r="H13" s="133" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="140"/>
-      <c r="J13" s="132">
+      <c r="I13" s="134"/>
+      <c r="J13" s="135">
         <v>45688</v>
       </c>
-      <c r="K13" s="133" t="s">
+      <c r="K13" s="136" t="s">
         <v>19</v>
       </c>
-      <c r="L13" s="133"/>
-      <c r="M13" s="133"/>
-      <c r="N13" s="133"/>
-      <c r="O13" s="132" t="s">
+      <c r="L13" s="136"/>
+      <c r="M13" s="136"/>
+      <c r="N13" s="136"/>
+      <c r="O13" s="135" t="s">
         <v>97</v>
       </c>
-      <c r="P13" s="133"/>
-      <c r="Q13" s="133"/>
-      <c r="R13" s="133"/>
-      <c r="S13" s="134"/>
-      <c r="T13" s="132">
+      <c r="P13" s="136"/>
+      <c r="Q13" s="136"/>
+      <c r="R13" s="136"/>
+      <c r="S13" s="137"/>
+      <c r="T13" s="135">
         <v>45747</v>
       </c>
-      <c r="U13" s="133" t="s">
+      <c r="U13" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="V13" s="133"/>
-      <c r="W13" s="133"/>
-      <c r="X13" s="134"/>
-      <c r="Y13" s="132">
+      <c r="V13" s="136"/>
+      <c r="W13" s="136"/>
+      <c r="X13" s="137"/>
+      <c r="Y13" s="135">
         <v>45777</v>
       </c>
-      <c r="Z13" s="133" t="s">
+      <c r="Z13" s="136" t="s">
         <v>21</v>
       </c>
-      <c r="AA13" s="133"/>
-      <c r="AB13" s="133"/>
-      <c r="AC13" s="134"/>
-      <c r="AD13" s="132">
+      <c r="AA13" s="136"/>
+      <c r="AB13" s="136"/>
+      <c r="AC13" s="137"/>
+      <c r="AD13" s="135">
         <v>45808</v>
       </c>
-      <c r="AE13" s="133" t="s">
+      <c r="AE13" s="136" t="s">
         <v>22</v>
       </c>
-      <c r="AF13" s="133"/>
-      <c r="AG13" s="133"/>
-      <c r="AH13" s="134"/>
-      <c r="AI13" s="132">
+      <c r="AF13" s="136"/>
+      <c r="AG13" s="136"/>
+      <c r="AH13" s="137"/>
+      <c r="AI13" s="135">
         <v>45838</v>
       </c>
-      <c r="AJ13" s="133" t="s">
+      <c r="AJ13" s="136" t="s">
         <v>23</v>
       </c>
-      <c r="AK13" s="133"/>
-      <c r="AL13" s="133"/>
-      <c r="AM13" s="134"/>
-      <c r="AN13" s="132">
+      <c r="AK13" s="136"/>
+      <c r="AL13" s="136"/>
+      <c r="AM13" s="137"/>
+      <c r="AN13" s="135">
         <v>45869</v>
       </c>
-      <c r="AO13" s="133" t="s">
+      <c r="AO13" s="136" t="s">
         <v>24</v>
       </c>
-      <c r="AP13" s="133"/>
-      <c r="AQ13" s="133"/>
-      <c r="AR13" s="134"/>
-      <c r="AS13" s="132">
+      <c r="AP13" s="136"/>
+      <c r="AQ13" s="136"/>
+      <c r="AR13" s="137"/>
+      <c r="AS13" s="135">
         <v>45900</v>
       </c>
-      <c r="AT13" s="133" t="s">
+      <c r="AT13" s="136" t="s">
         <v>25</v>
       </c>
-      <c r="AU13" s="133"/>
-      <c r="AV13" s="133"/>
-      <c r="AW13" s="134"/>
-      <c r="AX13" s="132">
+      <c r="AU13" s="136"/>
+      <c r="AV13" s="136"/>
+      <c r="AW13" s="137"/>
+      <c r="AX13" s="135">
         <v>45930</v>
       </c>
-      <c r="AY13" s="133" t="s">
+      <c r="AY13" s="136" t="s">
         <v>26</v>
       </c>
-      <c r="AZ13" s="133"/>
-      <c r="BA13" s="133"/>
-      <c r="BB13" s="134"/>
-      <c r="BC13" s="132">
+      <c r="AZ13" s="136"/>
+      <c r="BA13" s="136"/>
+      <c r="BB13" s="137"/>
+      <c r="BC13" s="135">
         <v>45961</v>
       </c>
-      <c r="BD13" s="133" t="s">
+      <c r="BD13" s="136" t="s">
         <v>27</v>
       </c>
-      <c r="BE13" s="133"/>
-      <c r="BF13" s="133"/>
-      <c r="BG13" s="134"/>
-      <c r="BH13" s="132">
+      <c r="BE13" s="136"/>
+      <c r="BF13" s="136"/>
+      <c r="BG13" s="137"/>
+      <c r="BH13" s="135">
         <v>45991</v>
       </c>
-      <c r="BI13" s="133" t="s">
+      <c r="BI13" s="136" t="s">
         <v>28</v>
       </c>
-      <c r="BJ13" s="133"/>
-      <c r="BK13" s="133"/>
-      <c r="BL13" s="134"/>
-      <c r="BM13" s="132">
+      <c r="BJ13" s="136"/>
+      <c r="BK13" s="136"/>
+      <c r="BL13" s="137"/>
+      <c r="BM13" s="135">
         <v>46022</v>
       </c>
-      <c r="BN13" s="133" t="s">
+      <c r="BN13" s="136" t="s">
         <v>29</v>
       </c>
-      <c r="BO13" s="133"/>
-      <c r="BP13" s="133"/>
-      <c r="BQ13" s="134"/>
+      <c r="BO13" s="136"/>
+      <c r="BP13" s="136"/>
+      <c r="BQ13" s="137"/>
       <c r="BR13" s="24">
         <f>SUM(BR15:BR24)</f>
         <v>0</v>
@@ -2368,7 +2409,7 @@
       <c r="Q14" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="R14" s="68" t="s">
+      <c r="R14" s="66" t="s">
         <v>47</v>
       </c>
       <c r="S14" s="35" t="s">
@@ -2383,7 +2424,7 @@
       <c r="V14" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="W14" s="68" t="s">
+      <c r="W14" s="66" t="s">
         <v>51</v>
       </c>
       <c r="X14" s="35" t="s">
@@ -2398,7 +2439,7 @@
       <c r="AA14" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="AB14" s="68" t="s">
+      <c r="AB14" s="66" t="s">
         <v>55</v>
       </c>
       <c r="AC14" s="35" t="s">
@@ -2413,7 +2454,7 @@
       <c r="AF14" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="AG14" s="68" t="s">
+      <c r="AG14" s="66" t="s">
         <v>58</v>
       </c>
       <c r="AH14" s="35" t="s">
@@ -2428,7 +2469,7 @@
       <c r="AK14" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="AL14" s="68" t="s">
+      <c r="AL14" s="66" t="s">
         <v>62</v>
       </c>
       <c r="AM14" s="35" t="s">
@@ -2443,7 +2484,7 @@
       <c r="AP14" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="AQ14" s="68" t="s">
+      <c r="AQ14" s="66" t="s">
         <v>66</v>
       </c>
       <c r="AR14" s="35" t="s">
@@ -2458,7 +2499,7 @@
       <c r="AU14" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="AV14" s="68" t="s">
+      <c r="AV14" s="66" t="s">
         <v>70</v>
       </c>
       <c r="AW14" s="35" t="s">
@@ -2473,7 +2514,7 @@
       <c r="AZ14" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="BA14" s="68" t="s">
+      <c r="BA14" s="66" t="s">
         <v>74</v>
       </c>
       <c r="BB14" s="35" t="s">
@@ -2488,7 +2529,7 @@
       <c r="BE14" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="BF14" s="68" t="s">
+      <c r="BF14" s="66" t="s">
         <v>78</v>
       </c>
       <c r="BG14" s="35" t="s">
@@ -2503,7 +2544,7 @@
       <c r="BJ14" s="34" t="s">
         <v>81</v>
       </c>
-      <c r="BK14" s="68" t="s">
+      <c r="BK14" s="66" t="s">
         <v>82</v>
       </c>
       <c r="BL14" s="35" t="s">
@@ -2518,7 +2559,7 @@
       <c r="BO14" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="BP14" s="68" t="s">
+      <c r="BP14" s="66" t="s">
         <v>86</v>
       </c>
       <c r="BQ14" s="35" t="s">
@@ -2534,1227 +2575,1259 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:73" x14ac:dyDescent="0.25">
-      <c r="A15" s="39"/>
-      <c r="B15" s="40" t="s">
+    <row r="15" spans="1:73" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="138" t="s">
+        <v>100</v>
+      </c>
+      <c r="B15" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="C15" s="69"/>
-      <c r="D15" s="69"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="42"/>
-      <c r="J15" s="43"/>
-      <c r="K15" s="41"/>
-      <c r="L15" s="41"/>
-      <c r="M15" s="44"/>
-      <c r="N15" s="44">
+      <c r="C15" s="139">
+        <v>45658</v>
+      </c>
+      <c r="D15" s="139">
+        <v>45838</v>
+      </c>
+      <c r="E15" s="140" t="s">
+        <v>101</v>
+      </c>
+      <c r="F15" s="140" t="s">
+        <v>102</v>
+      </c>
+      <c r="G15" s="141">
+        <v>108680</v>
+      </c>
+      <c r="H15" s="142" t="s">
+        <v>103</v>
+      </c>
+      <c r="I15" s="143" t="s">
+        <v>104</v>
+      </c>
+      <c r="J15" s="41"/>
+      <c r="K15" s="40"/>
+      <c r="L15" s="40"/>
+      <c r="M15" s="42"/>
+      <c r="N15" s="42">
         <f>L15-M15</f>
         <v>0</v>
       </c>
-      <c r="O15" s="43"/>
-      <c r="P15" s="41"/>
-      <c r="Q15" s="41"/>
-      <c r="R15" s="44"/>
-      <c r="S15" s="45">
+      <c r="O15" s="41"/>
+      <c r="P15" s="40"/>
+      <c r="Q15" s="40"/>
+      <c r="R15" s="42"/>
+      <c r="S15" s="43">
         <f t="shared" ref="S15:S20" si="1">Q15-R15</f>
         <v>0</v>
       </c>
-      <c r="T15" s="46"/>
-      <c r="U15" s="41"/>
-      <c r="V15" s="41"/>
-      <c r="W15" s="44"/>
-      <c r="X15" s="53">
+      <c r="T15" s="44"/>
+      <c r="U15" s="40"/>
+      <c r="V15" s="40"/>
+      <c r="W15" s="42"/>
+      <c r="X15" s="51">
         <f>V15-W15</f>
         <v>0</v>
       </c>
-      <c r="Y15" s="46"/>
-      <c r="Z15" s="41"/>
-      <c r="AA15" s="41"/>
-      <c r="AB15" s="44"/>
-      <c r="AC15" s="53">
+      <c r="Y15" s="44"/>
+      <c r="Z15" s="40"/>
+      <c r="AA15" s="40"/>
+      <c r="AB15" s="42"/>
+      <c r="AC15" s="51">
         <f>AA15-AB15</f>
         <v>0</v>
       </c>
-      <c r="AD15" s="46"/>
-      <c r="AE15" s="41"/>
-      <c r="AF15" s="41"/>
-      <c r="AG15" s="44"/>
-      <c r="AH15" s="53">
+      <c r="AD15" s="44"/>
+      <c r="AE15" s="40"/>
+      <c r="AF15" s="40"/>
+      <c r="AG15" s="42"/>
+      <c r="AH15" s="51">
         <f>AF15-AG15</f>
         <v>0</v>
       </c>
-      <c r="AI15" s="46"/>
-      <c r="AJ15" s="41"/>
-      <c r="AK15" s="41"/>
-      <c r="AL15" s="44"/>
-      <c r="AM15" s="53">
+      <c r="AI15" s="44"/>
+      <c r="AJ15" s="40"/>
+      <c r="AK15" s="40"/>
+      <c r="AL15" s="42"/>
+      <c r="AM15" s="51">
         <f>AK15-AL15</f>
         <v>0</v>
       </c>
-      <c r="AN15" s="46"/>
-      <c r="AO15" s="41"/>
-      <c r="AP15" s="41"/>
-      <c r="AQ15" s="44"/>
-      <c r="AR15" s="53">
+      <c r="AN15" s="44"/>
+      <c r="AO15" s="40"/>
+      <c r="AP15" s="40"/>
+      <c r="AQ15" s="42"/>
+      <c r="AR15" s="51">
         <f>AP15-AQ15</f>
         <v>0</v>
       </c>
-      <c r="AS15" s="46"/>
-      <c r="AT15" s="41"/>
-      <c r="AU15" s="41"/>
-      <c r="AV15" s="44"/>
-      <c r="AW15" s="53">
+      <c r="AS15" s="44"/>
+      <c r="AT15" s="40"/>
+      <c r="AU15" s="40"/>
+      <c r="AV15" s="42"/>
+      <c r="AW15" s="51">
         <f>AU15-AV15</f>
         <v>0</v>
       </c>
-      <c r="AX15" s="46"/>
-      <c r="AY15" s="41"/>
-      <c r="AZ15" s="41"/>
-      <c r="BA15" s="44"/>
-      <c r="BB15" s="53">
+      <c r="AX15" s="44"/>
+      <c r="AY15" s="40"/>
+      <c r="AZ15" s="40"/>
+      <c r="BA15" s="42"/>
+      <c r="BB15" s="51">
         <f>AZ15-BA15</f>
         <v>0</v>
       </c>
-      <c r="BC15" s="46"/>
-      <c r="BD15" s="41"/>
-      <c r="BE15" s="41"/>
-      <c r="BF15" s="44"/>
-      <c r="BG15" s="53">
+      <c r="BC15" s="44"/>
+      <c r="BD15" s="40"/>
+      <c r="BE15" s="40"/>
+      <c r="BF15" s="42"/>
+      <c r="BG15" s="51">
         <f>BE15-BF15</f>
         <v>0</v>
       </c>
-      <c r="BH15" s="46"/>
-      <c r="BI15" s="41"/>
-      <c r="BJ15" s="41"/>
-      <c r="BK15" s="44"/>
-      <c r="BL15" s="53">
+      <c r="BH15" s="44"/>
+      <c r="BI15" s="40"/>
+      <c r="BJ15" s="40"/>
+      <c r="BK15" s="42"/>
+      <c r="BL15" s="51">
         <f>BJ15-BK15</f>
         <v>0</v>
       </c>
-      <c r="BM15" s="46"/>
-      <c r="BN15" s="41"/>
-      <c r="BO15" s="41"/>
-      <c r="BP15" s="44"/>
-      <c r="BQ15" s="53">
+      <c r="BM15" s="44"/>
+      <c r="BN15" s="40"/>
+      <c r="BO15" s="40"/>
+      <c r="BP15" s="42"/>
+      <c r="BQ15" s="51">
         <f t="shared" ref="BQ15:BQ20" si="2">BO15-BP15</f>
         <v>0</v>
       </c>
-      <c r="BR15" s="43">
+      <c r="BR15" s="41">
         <f t="shared" ref="BR15:BR23" si="3">SUM(IF(M15&lt;&gt;"",M15,IF(L15&lt;&gt;"",L15,K15)),IF(R15&lt;&gt;"",R15,IF(Q15&lt;&gt;"",Q15,P15)),IF(W15&lt;&gt;"",W15,IF(V15&lt;&gt;"",V15,U15)),IF(AB15&lt;&gt;"",AB15,IF(AA15&lt;&gt;"",AA15,Z15)),IF(AG15&lt;&gt;"",AG15,IF(AF15&lt;&gt;"",AF15,AE15)),IF(AL15&lt;&gt;"",AL15,IF(AK15&lt;&gt;"",AK15,AJ15)),IF(AQ15&lt;&gt;"",AQ15,IF(AP15&lt;&gt;"",AP15,AO15)),IF(AV15&lt;&gt;"",AV15,IF(AU15&lt;&gt;"",AU15,AT15)),IF(BA15&lt;&gt;"",BA15,IF(AZ15&lt;&gt;"",AZ15,AY15)),IF(BF15&lt;&gt;"",BF15,IF(BE15&lt;&gt;"",BE15,BD15)),IF(BK15&lt;&gt;"",BK15,IF(BJ15&lt;&gt;"",BJ15,BI15)),IF(BP15&lt;&gt;"",BP15,IF(BO15&lt;&gt;"",BO15,BN15)))</f>
         <v>0</v>
       </c>
-      <c r="BS15" s="70"/>
-      <c r="BT15" s="71"/>
+      <c r="BS15" s="67"/>
+      <c r="BT15" s="68"/>
     </row>
-    <row r="16" spans="1:73" x14ac:dyDescent="0.25">
-      <c r="A16" s="47"/>
-      <c r="B16" s="48" t="s">
+    <row r="16" spans="1:73" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="45" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16" s="46" t="s">
         <v>99</v>
       </c>
-      <c r="C16" s="72"/>
-      <c r="D16" s="72"/>
-      <c r="E16" s="72"/>
-      <c r="F16" s="48"/>
-      <c r="G16" s="49"/>
-      <c r="H16" s="48"/>
-      <c r="I16" s="50"/>
-      <c r="J16" s="51"/>
-      <c r="K16" s="49"/>
-      <c r="L16" s="49"/>
-      <c r="M16" s="52"/>
-      <c r="N16" s="52">
+      <c r="C16" s="144">
+        <v>45658</v>
+      </c>
+      <c r="D16" s="144">
+        <v>45838</v>
+      </c>
+      <c r="E16" s="145" t="s">
+        <v>101</v>
+      </c>
+      <c r="F16" s="145" t="s">
+        <v>105</v>
+      </c>
+      <c r="G16" s="146">
+        <v>315000</v>
+      </c>
+      <c r="H16" s="147" t="s">
+        <v>106</v>
+      </c>
+      <c r="I16" s="148" t="s">
+        <v>104</v>
+      </c>
+      <c r="J16" s="49"/>
+      <c r="K16" s="47"/>
+      <c r="L16" s="47"/>
+      <c r="M16" s="50"/>
+      <c r="N16" s="50">
         <f t="shared" ref="N16:N20" si="4">L16-M16</f>
         <v>0</v>
       </c>
-      <c r="O16" s="51"/>
-      <c r="P16" s="49"/>
-      <c r="Q16" s="49"/>
-      <c r="R16" s="52"/>
-      <c r="S16" s="53">
+      <c r="O16" s="49"/>
+      <c r="P16" s="47"/>
+      <c r="Q16" s="47"/>
+      <c r="R16" s="50"/>
+      <c r="S16" s="51">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="T16" s="54"/>
-      <c r="U16" s="49"/>
-      <c r="V16" s="49"/>
-      <c r="W16" s="52"/>
-      <c r="X16" s="53">
+      <c r="T16" s="52"/>
+      <c r="U16" s="47"/>
+      <c r="V16" s="47"/>
+      <c r="W16" s="50"/>
+      <c r="X16" s="51">
         <f t="shared" ref="X16:X20" si="5">V16-W16</f>
         <v>0</v>
       </c>
-      <c r="Y16" s="54"/>
-      <c r="Z16" s="49"/>
-      <c r="AA16" s="49"/>
-      <c r="AB16" s="49"/>
-      <c r="AC16" s="53">
+      <c r="Y16" s="52"/>
+      <c r="Z16" s="47"/>
+      <c r="AA16" s="47"/>
+      <c r="AB16" s="47"/>
+      <c r="AC16" s="51">
         <f t="shared" ref="AC16:AC20" si="6">AA16-AB16</f>
         <v>0</v>
       </c>
-      <c r="AD16" s="54"/>
-      <c r="AE16" s="49"/>
-      <c r="AF16" s="49"/>
-      <c r="AG16" s="49"/>
-      <c r="AH16" s="53">
+      <c r="AD16" s="52"/>
+      <c r="AE16" s="47"/>
+      <c r="AF16" s="47"/>
+      <c r="AG16" s="47"/>
+      <c r="AH16" s="51">
         <f t="shared" ref="AH16:AH20" si="7">AF16-AG16</f>
         <v>0</v>
       </c>
-      <c r="AI16" s="54"/>
-      <c r="AJ16" s="49"/>
-      <c r="AK16" s="49"/>
-      <c r="AL16" s="49"/>
-      <c r="AM16" s="53">
+      <c r="AI16" s="52"/>
+      <c r="AJ16" s="47"/>
+      <c r="AK16" s="47"/>
+      <c r="AL16" s="47"/>
+      <c r="AM16" s="51">
         <f t="shared" ref="AM16:AM20" si="8">AK16-AL16</f>
         <v>0</v>
       </c>
-      <c r="AN16" s="54"/>
-      <c r="AO16" s="49"/>
-      <c r="AP16" s="49"/>
-      <c r="AQ16" s="49"/>
-      <c r="AR16" s="53">
+      <c r="AN16" s="52"/>
+      <c r="AO16" s="47"/>
+      <c r="AP16" s="47"/>
+      <c r="AQ16" s="47"/>
+      <c r="AR16" s="51">
         <f t="shared" ref="AR16:AR20" si="9">AP16-AQ16</f>
         <v>0</v>
       </c>
-      <c r="AS16" s="54"/>
-      <c r="AT16" s="49"/>
-      <c r="AU16" s="49"/>
-      <c r="AV16" s="49"/>
-      <c r="AW16" s="53">
+      <c r="AS16" s="52"/>
+      <c r="AT16" s="47"/>
+      <c r="AU16" s="47"/>
+      <c r="AV16" s="47"/>
+      <c r="AW16" s="51">
         <f t="shared" ref="AW16:AW20" si="10">AU16-AV16</f>
         <v>0</v>
       </c>
-      <c r="AX16" s="54"/>
-      <c r="AY16" s="49"/>
-      <c r="AZ16" s="49"/>
-      <c r="BA16" s="49"/>
-      <c r="BB16" s="53">
+      <c r="AX16" s="52"/>
+      <c r="AY16" s="47"/>
+      <c r="AZ16" s="47"/>
+      <c r="BA16" s="47"/>
+      <c r="BB16" s="51">
         <f t="shared" ref="BB16:BB20" si="11">AZ16-BA16</f>
         <v>0</v>
       </c>
-      <c r="BC16" s="54"/>
-      <c r="BD16" s="49"/>
-      <c r="BE16" s="49"/>
-      <c r="BF16" s="49"/>
-      <c r="BG16" s="53">
+      <c r="BC16" s="52"/>
+      <c r="BD16" s="47"/>
+      <c r="BE16" s="47"/>
+      <c r="BF16" s="47"/>
+      <c r="BG16" s="51">
         <f t="shared" ref="BG16:BG20" si="12">BE16-BF16</f>
         <v>0</v>
       </c>
-      <c r="BH16" s="54"/>
-      <c r="BI16" s="49"/>
-      <c r="BJ16" s="49"/>
-      <c r="BK16" s="49"/>
-      <c r="BL16" s="53">
+      <c r="BH16" s="52"/>
+      <c r="BI16" s="47"/>
+      <c r="BJ16" s="47"/>
+      <c r="BK16" s="47"/>
+      <c r="BL16" s="51">
         <f t="shared" ref="BL16:BL20" si="13">BJ16-BK16</f>
         <v>0</v>
       </c>
-      <c r="BM16" s="54"/>
-      <c r="BN16" s="49"/>
-      <c r="BO16" s="49"/>
-      <c r="BP16" s="49"/>
-      <c r="BQ16" s="53">
+      <c r="BM16" s="52"/>
+      <c r="BN16" s="47"/>
+      <c r="BO16" s="47"/>
+      <c r="BP16" s="47"/>
+      <c r="BQ16" s="51">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="BR16" s="51">
+      <c r="BR16" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="BS16" s="73"/>
-      <c r="BT16" s="74"/>
+      <c r="BS16" s="70"/>
+      <c r="BT16" s="71"/>
     </row>
     <row r="17" spans="1:72" x14ac:dyDescent="0.25">
-      <c r="A17" s="47"/>
-      <c r="B17" s="48"/>
-      <c r="C17" s="72"/>
-      <c r="D17" s="72"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="48"/>
-      <c r="G17" s="49"/>
-      <c r="H17" s="48"/>
-      <c r="I17" s="50"/>
-      <c r="J17" s="55"/>
-      <c r="K17" s="56"/>
-      <c r="L17" s="56"/>
-      <c r="M17" s="52"/>
-      <c r="N17" s="52">
+      <c r="A17" s="45"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="69"/>
+      <c r="D17" s="69"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="46"/>
+      <c r="G17" s="47"/>
+      <c r="H17" s="46"/>
+      <c r="I17" s="48"/>
+      <c r="J17" s="53"/>
+      <c r="K17" s="54"/>
+      <c r="L17" s="54"/>
+      <c r="M17" s="50"/>
+      <c r="N17" s="50">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="O17" s="55"/>
-      <c r="P17" s="49"/>
-      <c r="Q17" s="49"/>
-      <c r="R17" s="52"/>
-      <c r="S17" s="53">
+      <c r="O17" s="53"/>
+      <c r="P17" s="47"/>
+      <c r="Q17" s="47"/>
+      <c r="R17" s="50"/>
+      <c r="S17" s="51">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="T17" s="54"/>
-      <c r="U17" s="49"/>
-      <c r="V17" s="49"/>
-      <c r="W17" s="57"/>
-      <c r="X17" s="53">
+      <c r="T17" s="52"/>
+      <c r="U17" s="47"/>
+      <c r="V17" s="47"/>
+      <c r="W17" s="55"/>
+      <c r="X17" s="51">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Y17" s="54"/>
-      <c r="Z17" s="56"/>
-      <c r="AA17" s="56"/>
-      <c r="AB17" s="57"/>
-      <c r="AC17" s="53">
+      <c r="Y17" s="52"/>
+      <c r="Z17" s="54"/>
+      <c r="AA17" s="54"/>
+      <c r="AB17" s="55"/>
+      <c r="AC17" s="51">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="AD17" s="54"/>
-      <c r="AE17" s="56"/>
-      <c r="AF17" s="56"/>
-      <c r="AG17" s="57"/>
-      <c r="AH17" s="53">
+      <c r="AD17" s="52"/>
+      <c r="AE17" s="54"/>
+      <c r="AF17" s="54"/>
+      <c r="AG17" s="55"/>
+      <c r="AH17" s="51">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AI17" s="54"/>
-      <c r="AJ17" s="56"/>
-      <c r="AK17" s="56"/>
-      <c r="AL17" s="57"/>
-      <c r="AM17" s="53">
+      <c r="AI17" s="52"/>
+      <c r="AJ17" s="54"/>
+      <c r="AK17" s="54"/>
+      <c r="AL17" s="55"/>
+      <c r="AM17" s="51">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="AN17" s="54"/>
-      <c r="AO17" s="56"/>
-      <c r="AP17" s="56"/>
-      <c r="AQ17" s="57"/>
-      <c r="AR17" s="53">
+      <c r="AN17" s="52"/>
+      <c r="AO17" s="54"/>
+      <c r="AP17" s="54"/>
+      <c r="AQ17" s="55"/>
+      <c r="AR17" s="51">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AS17" s="54"/>
-      <c r="AT17" s="56"/>
-      <c r="AU17" s="56"/>
-      <c r="AV17" s="57"/>
-      <c r="AW17" s="53">
+      <c r="AS17" s="52"/>
+      <c r="AT17" s="54"/>
+      <c r="AU17" s="54"/>
+      <c r="AV17" s="55"/>
+      <c r="AW17" s="51">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="AX17" s="54"/>
-      <c r="AY17" s="56"/>
-      <c r="AZ17" s="56"/>
-      <c r="BA17" s="57"/>
-      <c r="BB17" s="53">
+      <c r="AX17" s="52"/>
+      <c r="AY17" s="54"/>
+      <c r="AZ17" s="54"/>
+      <c r="BA17" s="55"/>
+      <c r="BB17" s="51">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="BC17" s="54"/>
-      <c r="BD17" s="56"/>
-      <c r="BE17" s="56"/>
-      <c r="BF17" s="57"/>
-      <c r="BG17" s="53">
+      <c r="BC17" s="52"/>
+      <c r="BD17" s="54"/>
+      <c r="BE17" s="54"/>
+      <c r="BF17" s="55"/>
+      <c r="BG17" s="51">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="BH17" s="54"/>
-      <c r="BI17" s="56"/>
-      <c r="BJ17" s="56"/>
-      <c r="BK17" s="57"/>
-      <c r="BL17" s="53">
+      <c r="BH17" s="52"/>
+      <c r="BI17" s="54"/>
+      <c r="BJ17" s="54"/>
+      <c r="BK17" s="55"/>
+      <c r="BL17" s="51">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="BM17" s="54"/>
-      <c r="BN17" s="56"/>
-      <c r="BO17" s="56"/>
-      <c r="BP17" s="57"/>
-      <c r="BQ17" s="53">
+      <c r="BM17" s="52"/>
+      <c r="BN17" s="54"/>
+      <c r="BO17" s="54"/>
+      <c r="BP17" s="55"/>
+      <c r="BQ17" s="51">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="BR17" s="51">
+      <c r="BR17" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="BS17" s="73"/>
-      <c r="BT17" s="74"/>
+      <c r="BS17" s="70"/>
+      <c r="BT17" s="71"/>
     </row>
     <row r="18" spans="1:72" x14ac:dyDescent="0.25">
-      <c r="A18" s="47"/>
-      <c r="B18" s="48"/>
-      <c r="C18" s="72"/>
-      <c r="D18" s="72"/>
-      <c r="E18" s="48"/>
-      <c r="F18" s="48"/>
-      <c r="G18" s="49"/>
-      <c r="H18" s="48"/>
-      <c r="I18" s="50"/>
-      <c r="J18" s="51"/>
-      <c r="K18" s="49"/>
-      <c r="L18" s="49"/>
-      <c r="M18" s="52"/>
-      <c r="N18" s="52">
+      <c r="A18" s="45"/>
+      <c r="B18" s="46"/>
+      <c r="C18" s="69"/>
+      <c r="D18" s="69"/>
+      <c r="E18" s="46"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="47"/>
+      <c r="H18" s="46"/>
+      <c r="I18" s="48"/>
+      <c r="J18" s="49"/>
+      <c r="K18" s="47"/>
+      <c r="L18" s="47"/>
+      <c r="M18" s="50"/>
+      <c r="N18" s="50">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="O18" s="51"/>
-      <c r="P18" s="49"/>
-      <c r="Q18" s="49"/>
-      <c r="R18" s="52"/>
-      <c r="S18" s="53">
+      <c r="O18" s="49"/>
+      <c r="P18" s="47"/>
+      <c r="Q18" s="47"/>
+      <c r="R18" s="50"/>
+      <c r="S18" s="51">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="T18" s="54"/>
-      <c r="U18" s="49"/>
-      <c r="V18" s="49"/>
-      <c r="W18" s="52"/>
-      <c r="X18" s="53">
+      <c r="T18" s="52"/>
+      <c r="U18" s="47"/>
+      <c r="V18" s="47"/>
+      <c r="W18" s="50"/>
+      <c r="X18" s="51">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Y18" s="54"/>
-      <c r="Z18" s="49"/>
-      <c r="AA18" s="49"/>
-      <c r="AB18" s="52"/>
-      <c r="AC18" s="53">
+      <c r="Y18" s="52"/>
+      <c r="Z18" s="47"/>
+      <c r="AA18" s="47"/>
+      <c r="AB18" s="50"/>
+      <c r="AC18" s="51">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="AD18" s="54"/>
-      <c r="AE18" s="49"/>
-      <c r="AF18" s="49"/>
-      <c r="AG18" s="52"/>
-      <c r="AH18" s="53">
+      <c r="AD18" s="52"/>
+      <c r="AE18" s="47"/>
+      <c r="AF18" s="47"/>
+      <c r="AG18" s="50"/>
+      <c r="AH18" s="51">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AI18" s="54"/>
-      <c r="AJ18" s="49"/>
-      <c r="AK18" s="49"/>
-      <c r="AL18" s="52"/>
-      <c r="AM18" s="53">
+      <c r="AI18" s="52"/>
+      <c r="AJ18" s="47"/>
+      <c r="AK18" s="47"/>
+      <c r="AL18" s="50"/>
+      <c r="AM18" s="51">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="AN18" s="54"/>
-      <c r="AO18" s="49"/>
-      <c r="AP18" s="49"/>
-      <c r="AQ18" s="52"/>
-      <c r="AR18" s="53">
+      <c r="AN18" s="52"/>
+      <c r="AO18" s="47"/>
+      <c r="AP18" s="47"/>
+      <c r="AQ18" s="50"/>
+      <c r="AR18" s="51">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AS18" s="54"/>
-      <c r="AT18" s="49"/>
-      <c r="AU18" s="49"/>
-      <c r="AV18" s="52"/>
-      <c r="AW18" s="53">
+      <c r="AS18" s="52"/>
+      <c r="AT18" s="47"/>
+      <c r="AU18" s="47"/>
+      <c r="AV18" s="50"/>
+      <c r="AW18" s="51">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="AX18" s="54"/>
-      <c r="AY18" s="49"/>
-      <c r="AZ18" s="49"/>
-      <c r="BA18" s="52"/>
-      <c r="BB18" s="53">
+      <c r="AX18" s="52"/>
+      <c r="AY18" s="47"/>
+      <c r="AZ18" s="47"/>
+      <c r="BA18" s="50"/>
+      <c r="BB18" s="51">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="BC18" s="54"/>
-      <c r="BD18" s="49"/>
-      <c r="BE18" s="49"/>
-      <c r="BF18" s="52"/>
-      <c r="BG18" s="53">
+      <c r="BC18" s="52"/>
+      <c r="BD18" s="47"/>
+      <c r="BE18" s="47"/>
+      <c r="BF18" s="50"/>
+      <c r="BG18" s="51">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="BH18" s="54"/>
-      <c r="BI18" s="49"/>
-      <c r="BJ18" s="49"/>
-      <c r="BK18" s="52"/>
-      <c r="BL18" s="53">
+      <c r="BH18" s="52"/>
+      <c r="BI18" s="47"/>
+      <c r="BJ18" s="47"/>
+      <c r="BK18" s="50"/>
+      <c r="BL18" s="51">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="BM18" s="54"/>
-      <c r="BN18" s="49"/>
-      <c r="BO18" s="49"/>
-      <c r="BP18" s="52"/>
-      <c r="BQ18" s="53">
+      <c r="BM18" s="52"/>
+      <c r="BN18" s="47"/>
+      <c r="BO18" s="47"/>
+      <c r="BP18" s="50"/>
+      <c r="BQ18" s="51">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="BR18" s="51">
+      <c r="BR18" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="BS18" s="73"/>
-      <c r="BT18" s="74"/>
+      <c r="BS18" s="70"/>
+      <c r="BT18" s="71"/>
     </row>
     <row r="19" spans="1:72" x14ac:dyDescent="0.25">
-      <c r="A19" s="75"/>
-      <c r="C19" s="72"/>
-      <c r="D19" s="72"/>
-      <c r="E19" s="48"/>
-      <c r="F19" s="48"/>
-      <c r="G19" s="49"/>
-      <c r="H19" s="48"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="51"/>
-      <c r="K19" s="49"/>
-      <c r="L19" s="49"/>
-      <c r="M19" s="52"/>
-      <c r="N19" s="52">
+      <c r="A19" s="72"/>
+      <c r="C19" s="69"/>
+      <c r="D19" s="69"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="47"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="48"/>
+      <c r="J19" s="49"/>
+      <c r="K19" s="47"/>
+      <c r="L19" s="47"/>
+      <c r="M19" s="50"/>
+      <c r="N19" s="50">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="O19" s="51"/>
-      <c r="P19" s="49"/>
-      <c r="Q19" s="49"/>
-      <c r="R19" s="52"/>
-      <c r="S19" s="53">
+      <c r="O19" s="49"/>
+      <c r="P19" s="47"/>
+      <c r="Q19" s="47"/>
+      <c r="R19" s="50"/>
+      <c r="S19" s="51">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="T19" s="54"/>
-      <c r="U19" s="49"/>
-      <c r="V19" s="49"/>
-      <c r="W19" s="52"/>
-      <c r="X19" s="53">
+      <c r="T19" s="52"/>
+      <c r="U19" s="47"/>
+      <c r="V19" s="47"/>
+      <c r="W19" s="50"/>
+      <c r="X19" s="51">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Y19" s="54"/>
-      <c r="Z19" s="49"/>
-      <c r="AA19" s="49"/>
-      <c r="AB19" s="49"/>
-      <c r="AC19" s="53">
+      <c r="Y19" s="52"/>
+      <c r="Z19" s="47"/>
+      <c r="AA19" s="47"/>
+      <c r="AB19" s="47"/>
+      <c r="AC19" s="51">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="AD19" s="54"/>
-      <c r="AE19" s="49"/>
-      <c r="AF19" s="49"/>
-      <c r="AG19" s="49"/>
-      <c r="AH19" s="53">
+      <c r="AD19" s="52"/>
+      <c r="AE19" s="47"/>
+      <c r="AF19" s="47"/>
+      <c r="AG19" s="47"/>
+      <c r="AH19" s="51">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AI19" s="54"/>
-      <c r="AJ19" s="49"/>
-      <c r="AK19" s="49"/>
-      <c r="AL19" s="49"/>
-      <c r="AM19" s="53">
+      <c r="AI19" s="52"/>
+      <c r="AJ19" s="47"/>
+      <c r="AK19" s="47"/>
+      <c r="AL19" s="47"/>
+      <c r="AM19" s="51">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="AN19" s="54"/>
-      <c r="AO19" s="49"/>
-      <c r="AP19" s="49"/>
-      <c r="AQ19" s="49"/>
-      <c r="AR19" s="53">
+      <c r="AN19" s="52"/>
+      <c r="AO19" s="47"/>
+      <c r="AP19" s="47"/>
+      <c r="AQ19" s="47"/>
+      <c r="AR19" s="51">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AS19" s="54"/>
-      <c r="AT19" s="49"/>
-      <c r="AU19" s="49"/>
-      <c r="AV19" s="49"/>
-      <c r="AW19" s="53">
+      <c r="AS19" s="52"/>
+      <c r="AT19" s="47"/>
+      <c r="AU19" s="47"/>
+      <c r="AV19" s="47"/>
+      <c r="AW19" s="51">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="AX19" s="54"/>
-      <c r="AY19" s="49"/>
-      <c r="AZ19" s="49"/>
-      <c r="BA19" s="49"/>
-      <c r="BB19" s="53">
+      <c r="AX19" s="52"/>
+      <c r="AY19" s="47"/>
+      <c r="AZ19" s="47"/>
+      <c r="BA19" s="47"/>
+      <c r="BB19" s="51">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="BC19" s="54"/>
-      <c r="BD19" s="49"/>
-      <c r="BE19" s="49"/>
-      <c r="BF19" s="49"/>
-      <c r="BG19" s="53">
+      <c r="BC19" s="52"/>
+      <c r="BD19" s="47"/>
+      <c r="BE19" s="47"/>
+      <c r="BF19" s="47"/>
+      <c r="BG19" s="51">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="BH19" s="54"/>
-      <c r="BI19" s="49"/>
-      <c r="BJ19" s="49"/>
-      <c r="BK19" s="49"/>
-      <c r="BL19" s="53">
+      <c r="BH19" s="52"/>
+      <c r="BI19" s="47"/>
+      <c r="BJ19" s="47"/>
+      <c r="BK19" s="47"/>
+      <c r="BL19" s="51">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="BM19" s="54"/>
-      <c r="BN19" s="49"/>
-      <c r="BO19" s="49"/>
-      <c r="BP19" s="49"/>
-      <c r="BQ19" s="53">
+      <c r="BM19" s="52"/>
+      <c r="BN19" s="47"/>
+      <c r="BO19" s="47"/>
+      <c r="BP19" s="47"/>
+      <c r="BQ19" s="51">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="BR19" s="51">
+      <c r="BR19" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="BS19" s="73"/>
-      <c r="BT19" s="74"/>
+      <c r="BS19" s="70"/>
+      <c r="BT19" s="71"/>
     </row>
     <row r="20" spans="1:72" x14ac:dyDescent="0.25">
-      <c r="A20" s="47"/>
-      <c r="B20" s="48"/>
-      <c r="C20" s="72"/>
-      <c r="D20" s="72"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="49"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="50"/>
-      <c r="J20" s="51"/>
-      <c r="K20" s="49"/>
-      <c r="L20" s="49"/>
-      <c r="M20" s="52"/>
-      <c r="N20" s="52">
+      <c r="A20" s="45"/>
+      <c r="B20" s="46"/>
+      <c r="C20" s="69"/>
+      <c r="D20" s="69"/>
+      <c r="E20" s="46"/>
+      <c r="F20" s="46"/>
+      <c r="G20" s="47"/>
+      <c r="H20" s="46"/>
+      <c r="I20" s="48"/>
+      <c r="J20" s="49"/>
+      <c r="K20" s="47"/>
+      <c r="L20" s="47"/>
+      <c r="M20" s="50"/>
+      <c r="N20" s="50">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="O20" s="51"/>
-      <c r="P20" s="49"/>
-      <c r="Q20" s="49"/>
-      <c r="R20" s="52"/>
-      <c r="S20" s="53">
+      <c r="O20" s="49"/>
+      <c r="P20" s="47"/>
+      <c r="Q20" s="47"/>
+      <c r="R20" s="50"/>
+      <c r="S20" s="51">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="T20" s="54"/>
-      <c r="U20" s="49"/>
-      <c r="V20" s="49"/>
-      <c r="W20" s="52"/>
-      <c r="X20" s="53">
+      <c r="T20" s="52"/>
+      <c r="U20" s="47"/>
+      <c r="V20" s="47"/>
+      <c r="W20" s="50"/>
+      <c r="X20" s="51">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Y20" s="54"/>
-      <c r="Z20" s="49"/>
-      <c r="AA20" s="49"/>
-      <c r="AB20" s="52"/>
-      <c r="AC20" s="53">
+      <c r="Y20" s="52"/>
+      <c r="Z20" s="47"/>
+      <c r="AA20" s="47"/>
+      <c r="AB20" s="50"/>
+      <c r="AC20" s="51">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="AD20" s="54"/>
-      <c r="AE20" s="49"/>
-      <c r="AF20" s="49"/>
-      <c r="AG20" s="52"/>
-      <c r="AH20" s="53">
+      <c r="AD20" s="52"/>
+      <c r="AE20" s="47"/>
+      <c r="AF20" s="47"/>
+      <c r="AG20" s="50"/>
+      <c r="AH20" s="51">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AI20" s="54"/>
-      <c r="AJ20" s="49"/>
-      <c r="AK20" s="49"/>
-      <c r="AL20" s="52"/>
-      <c r="AM20" s="53">
+      <c r="AI20" s="52"/>
+      <c r="AJ20" s="47"/>
+      <c r="AK20" s="47"/>
+      <c r="AL20" s="50"/>
+      <c r="AM20" s="51">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="AN20" s="54"/>
-      <c r="AO20" s="49"/>
-      <c r="AP20" s="49"/>
-      <c r="AQ20" s="52"/>
-      <c r="AR20" s="53">
+      <c r="AN20" s="52"/>
+      <c r="AO20" s="47"/>
+      <c r="AP20" s="47"/>
+      <c r="AQ20" s="50"/>
+      <c r="AR20" s="51">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AS20" s="54"/>
-      <c r="AT20" s="49"/>
-      <c r="AU20" s="49"/>
-      <c r="AV20" s="52"/>
-      <c r="AW20" s="53">
+      <c r="AS20" s="52"/>
+      <c r="AT20" s="47"/>
+      <c r="AU20" s="47"/>
+      <c r="AV20" s="50"/>
+      <c r="AW20" s="51">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="AX20" s="54"/>
-      <c r="AY20" s="49"/>
-      <c r="AZ20" s="49"/>
-      <c r="BA20" s="52"/>
-      <c r="BB20" s="53">
+      <c r="AX20" s="52"/>
+      <c r="AY20" s="47"/>
+      <c r="AZ20" s="47"/>
+      <c r="BA20" s="50"/>
+      <c r="BB20" s="51">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="BC20" s="54"/>
-      <c r="BD20" s="49"/>
-      <c r="BE20" s="49"/>
-      <c r="BF20" s="52"/>
-      <c r="BG20" s="53">
+      <c r="BC20" s="52"/>
+      <c r="BD20" s="47"/>
+      <c r="BE20" s="47"/>
+      <c r="BF20" s="50"/>
+      <c r="BG20" s="51">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="BH20" s="54"/>
-      <c r="BI20" s="49"/>
-      <c r="BJ20" s="49"/>
-      <c r="BK20" s="52"/>
-      <c r="BL20" s="53">
+      <c r="BH20" s="52"/>
+      <c r="BI20" s="47"/>
+      <c r="BJ20" s="47"/>
+      <c r="BK20" s="50"/>
+      <c r="BL20" s="51">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="BM20" s="54"/>
-      <c r="BN20" s="49"/>
-      <c r="BO20" s="49"/>
-      <c r="BP20" s="52"/>
-      <c r="BQ20" s="53">
+      <c r="BM20" s="52"/>
+      <c r="BN20" s="47"/>
+      <c r="BO20" s="47"/>
+      <c r="BP20" s="50"/>
+      <c r="BQ20" s="51">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="BR20" s="51">
+      <c r="BR20" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="BS20" s="73"/>
-      <c r="BT20" s="74"/>
+      <c r="BS20" s="70"/>
+      <c r="BT20" s="71"/>
     </row>
     <row r="21" spans="1:72" x14ac:dyDescent="0.25">
-      <c r="A21" s="47"/>
-      <c r="B21" s="48"/>
-      <c r="C21" s="72"/>
-      <c r="D21" s="72"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
-      <c r="G21" s="49"/>
-      <c r="H21" s="48"/>
-      <c r="I21" s="50"/>
-      <c r="J21" s="51"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="49"/>
-      <c r="M21" s="52"/>
-      <c r="N21" s="52"/>
-      <c r="O21" s="51"/>
-      <c r="P21" s="49"/>
-      <c r="Q21" s="49"/>
-      <c r="R21" s="52"/>
-      <c r="S21" s="53"/>
-      <c r="T21" s="54"/>
-      <c r="U21" s="49"/>
-      <c r="V21" s="49"/>
-      <c r="W21" s="52"/>
-      <c r="X21" s="53"/>
-      <c r="Y21" s="54"/>
-      <c r="Z21" s="49"/>
-      <c r="AA21" s="49"/>
-      <c r="AB21" s="52"/>
-      <c r="AC21" s="53"/>
-      <c r="AD21" s="54"/>
-      <c r="AE21" s="49"/>
-      <c r="AF21" s="49"/>
-      <c r="AG21" s="52"/>
-      <c r="AH21" s="53"/>
-      <c r="AI21" s="54"/>
-      <c r="AJ21" s="49"/>
-      <c r="AK21" s="49"/>
-      <c r="AL21" s="52"/>
-      <c r="AM21" s="53"/>
-      <c r="AN21" s="54"/>
-      <c r="AO21" s="49"/>
-      <c r="AP21" s="49"/>
-      <c r="AQ21" s="52"/>
-      <c r="AR21" s="53"/>
-      <c r="AS21" s="54"/>
-      <c r="AT21" s="49"/>
-      <c r="AU21" s="49"/>
-      <c r="AV21" s="52"/>
-      <c r="AW21" s="53"/>
-      <c r="AX21" s="54"/>
-      <c r="AY21" s="49"/>
-      <c r="AZ21" s="49"/>
-      <c r="BA21" s="52"/>
-      <c r="BB21" s="53"/>
-      <c r="BC21" s="54"/>
-      <c r="BD21" s="49"/>
-      <c r="BE21" s="49"/>
-      <c r="BF21" s="52"/>
-      <c r="BG21" s="53"/>
-      <c r="BH21" s="54"/>
-      <c r="BI21" s="49"/>
-      <c r="BJ21" s="49"/>
-      <c r="BK21" s="52"/>
-      <c r="BL21" s="53"/>
-      <c r="BM21" s="54"/>
-      <c r="BN21" s="49"/>
-      <c r="BO21" s="49"/>
-      <c r="BP21" s="52"/>
-      <c r="BQ21" s="53"/>
-      <c r="BR21" s="51"/>
-      <c r="BS21" s="73"/>
-      <c r="BT21" s="74"/>
+      <c r="A21" s="45"/>
+      <c r="B21" s="46"/>
+      <c r="C21" s="69"/>
+      <c r="D21" s="69"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="47"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="48"/>
+      <c r="J21" s="49"/>
+      <c r="K21" s="47"/>
+      <c r="L21" s="47"/>
+      <c r="M21" s="50"/>
+      <c r="N21" s="50"/>
+      <c r="O21" s="49"/>
+      <c r="P21" s="47"/>
+      <c r="Q21" s="47"/>
+      <c r="R21" s="50"/>
+      <c r="S21" s="51"/>
+      <c r="T21" s="52"/>
+      <c r="U21" s="47"/>
+      <c r="V21" s="47"/>
+      <c r="W21" s="50"/>
+      <c r="X21" s="51"/>
+      <c r="Y21" s="52"/>
+      <c r="Z21" s="47"/>
+      <c r="AA21" s="47"/>
+      <c r="AB21" s="50"/>
+      <c r="AC21" s="51"/>
+      <c r="AD21" s="52"/>
+      <c r="AE21" s="47"/>
+      <c r="AF21" s="47"/>
+      <c r="AG21" s="50"/>
+      <c r="AH21" s="51"/>
+      <c r="AI21" s="52"/>
+      <c r="AJ21" s="47"/>
+      <c r="AK21" s="47"/>
+      <c r="AL21" s="50"/>
+      <c r="AM21" s="51"/>
+      <c r="AN21" s="52"/>
+      <c r="AO21" s="47"/>
+      <c r="AP21" s="47"/>
+      <c r="AQ21" s="50"/>
+      <c r="AR21" s="51"/>
+      <c r="AS21" s="52"/>
+      <c r="AT21" s="47"/>
+      <c r="AU21" s="47"/>
+      <c r="AV21" s="50"/>
+      <c r="AW21" s="51"/>
+      <c r="AX21" s="52"/>
+      <c r="AY21" s="47"/>
+      <c r="AZ21" s="47"/>
+      <c r="BA21" s="50"/>
+      <c r="BB21" s="51"/>
+      <c r="BC21" s="52"/>
+      <c r="BD21" s="47"/>
+      <c r="BE21" s="47"/>
+      <c r="BF21" s="50"/>
+      <c r="BG21" s="51"/>
+      <c r="BH21" s="52"/>
+      <c r="BI21" s="47"/>
+      <c r="BJ21" s="47"/>
+      <c r="BK21" s="50"/>
+      <c r="BL21" s="51"/>
+      <c r="BM21" s="52"/>
+      <c r="BN21" s="47"/>
+      <c r="BO21" s="47"/>
+      <c r="BP21" s="50"/>
+      <c r="BQ21" s="51"/>
+      <c r="BR21" s="49"/>
+      <c r="BS21" s="70"/>
+      <c r="BT21" s="71"/>
     </row>
     <row r="22" spans="1:72" x14ac:dyDescent="0.25">
-      <c r="A22" s="99" t="s">
+      <c r="A22" s="96" t="s">
         <v>90</v>
       </c>
-      <c r="B22" s="100"/>
-      <c r="C22" s="101"/>
-      <c r="D22" s="101"/>
-      <c r="E22" s="100"/>
-      <c r="F22" s="100"/>
-      <c r="G22" s="102"/>
-      <c r="H22" s="100"/>
-      <c r="I22" s="103"/>
-      <c r="J22" s="104"/>
-      <c r="K22" s="102"/>
-      <c r="L22" s="102"/>
-      <c r="M22" s="105"/>
-      <c r="N22" s="105" t="str">
+      <c r="B22" s="97"/>
+      <c r="C22" s="98"/>
+      <c r="D22" s="98"/>
+      <c r="E22" s="97"/>
+      <c r="F22" s="97"/>
+      <c r="G22" s="99"/>
+      <c r="H22" s="97"/>
+      <c r="I22" s="100"/>
+      <c r="J22" s="101"/>
+      <c r="K22" s="99"/>
+      <c r="L22" s="99"/>
+      <c r="M22" s="102"/>
+      <c r="N22" s="102" t="str">
         <f>IF(OR(L22="",M22=""),"",L22-M22)</f>
         <v/>
       </c>
-      <c r="O22" s="104"/>
-      <c r="P22" s="102"/>
-      <c r="Q22" s="102"/>
-      <c r="R22" s="105"/>
-      <c r="S22" s="106" t="str">
+      <c r="O22" s="101"/>
+      <c r="P22" s="99"/>
+      <c r="Q22" s="99"/>
+      <c r="R22" s="102"/>
+      <c r="S22" s="103" t="str">
         <f t="shared" ref="S22:S24" si="14">IF(OR(Q22="",R22=""),"",Q22-R22)</f>
         <v/>
       </c>
-      <c r="T22" s="107"/>
-      <c r="U22" s="102"/>
-      <c r="V22" s="102"/>
-      <c r="W22" s="105"/>
-      <c r="X22" s="106" t="str">
+      <c r="T22" s="104"/>
+      <c r="U22" s="99"/>
+      <c r="V22" s="99"/>
+      <c r="W22" s="102"/>
+      <c r="X22" s="103" t="str">
         <f t="shared" ref="X22:X24" si="15">IF(OR(V22="",W22=""),"",V22-W22)</f>
         <v/>
       </c>
-      <c r="Y22" s="107"/>
-      <c r="Z22" s="102"/>
-      <c r="AA22" s="102"/>
-      <c r="AB22" s="105"/>
-      <c r="AC22" s="106" t="str">
+      <c r="Y22" s="104"/>
+      <c r="Z22" s="99"/>
+      <c r="AA22" s="99"/>
+      <c r="AB22" s="102"/>
+      <c r="AC22" s="103" t="str">
         <f t="shared" ref="AC22:AC24" si="16">IF(OR(AA22="",AB22=""),"",AA22-AB22)</f>
         <v/>
       </c>
-      <c r="AD22" s="107"/>
-      <c r="AE22" s="102"/>
-      <c r="AF22" s="102"/>
-      <c r="AG22" s="105"/>
-      <c r="AH22" s="106" t="str">
+      <c r="AD22" s="104"/>
+      <c r="AE22" s="99"/>
+      <c r="AF22" s="99"/>
+      <c r="AG22" s="102"/>
+      <c r="AH22" s="103" t="str">
         <f t="shared" ref="AH22:AH24" si="17">IF(OR(AF22="",AG22=""),"",AF22-AG22)</f>
         <v/>
       </c>
-      <c r="AI22" s="107"/>
-      <c r="AJ22" s="102"/>
-      <c r="AK22" s="102"/>
-      <c r="AL22" s="105"/>
-      <c r="AM22" s="106" t="str">
+      <c r="AI22" s="104"/>
+      <c r="AJ22" s="99"/>
+      <c r="AK22" s="99"/>
+      <c r="AL22" s="102"/>
+      <c r="AM22" s="103" t="str">
         <f t="shared" ref="AM22:AM24" si="18">IF(OR(AK22="",AL22=""),"",AK22-AL22)</f>
         <v/>
       </c>
-      <c r="AN22" s="107"/>
-      <c r="AO22" s="102"/>
-      <c r="AP22" s="102"/>
-      <c r="AQ22" s="105"/>
-      <c r="AR22" s="106" t="str">
+      <c r="AN22" s="104"/>
+      <c r="AO22" s="99"/>
+      <c r="AP22" s="99"/>
+      <c r="AQ22" s="102"/>
+      <c r="AR22" s="103" t="str">
         <f t="shared" ref="AR22:AR24" si="19">IF(OR(AP22="",AQ22=""),"",AP22-AQ22)</f>
         <v/>
       </c>
-      <c r="AS22" s="107"/>
-      <c r="AT22" s="102"/>
-      <c r="AU22" s="102"/>
-      <c r="AV22" s="105"/>
-      <c r="AW22" s="106" t="str">
+      <c r="AS22" s="104"/>
+      <c r="AT22" s="99"/>
+      <c r="AU22" s="99"/>
+      <c r="AV22" s="102"/>
+      <c r="AW22" s="103" t="str">
         <f t="shared" ref="AW22:AW24" si="20">IF(OR(AU22="",AV22=""),"",AU22-AV22)</f>
         <v/>
       </c>
-      <c r="AX22" s="107"/>
-      <c r="AY22" s="102"/>
-      <c r="AZ22" s="102"/>
-      <c r="BA22" s="105"/>
-      <c r="BB22" s="106" t="str">
+      <c r="AX22" s="104"/>
+      <c r="AY22" s="99"/>
+      <c r="AZ22" s="99"/>
+      <c r="BA22" s="102"/>
+      <c r="BB22" s="103" t="str">
         <f t="shared" ref="BB22:BB24" si="21">IF(OR(AZ22="",BA22=""),"",AZ22-BA22)</f>
         <v/>
       </c>
-      <c r="BC22" s="107"/>
-      <c r="BD22" s="102"/>
-      <c r="BE22" s="102"/>
-      <c r="BF22" s="105"/>
-      <c r="BG22" s="106" t="str">
+      <c r="BC22" s="104"/>
+      <c r="BD22" s="99"/>
+      <c r="BE22" s="99"/>
+      <c r="BF22" s="102"/>
+      <c r="BG22" s="103" t="str">
         <f t="shared" ref="BG22:BG24" si="22">IF(OR(BE22="",BF22=""),"",BE22-BF22)</f>
         <v/>
       </c>
-      <c r="BH22" s="107"/>
-      <c r="BI22" s="102"/>
-      <c r="BJ22" s="102"/>
-      <c r="BK22" s="105"/>
-      <c r="BL22" s="106" t="str">
+      <c r="BH22" s="104"/>
+      <c r="BI22" s="99"/>
+      <c r="BJ22" s="99"/>
+      <c r="BK22" s="102"/>
+      <c r="BL22" s="103" t="str">
         <f t="shared" ref="BL22:BL24" si="23">IF(OR(BJ22="",BK22=""),"",BJ22-BK22)</f>
         <v/>
       </c>
-      <c r="BM22" s="107"/>
-      <c r="BN22" s="102"/>
-      <c r="BO22" s="102"/>
-      <c r="BP22" s="105"/>
-      <c r="BQ22" s="106" t="str">
+      <c r="BM22" s="104"/>
+      <c r="BN22" s="99"/>
+      <c r="BO22" s="99"/>
+      <c r="BP22" s="102"/>
+      <c r="BQ22" s="103" t="str">
         <f t="shared" ref="BQ22:BQ24" si="24">IF(OR(BO22="",BP22=""),"",BO22-BP22)</f>
         <v/>
       </c>
-      <c r="BR22" s="104">
+      <c r="BR22" s="101">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="BS22" s="108"/>
-      <c r="BT22" s="109"/>
+      <c r="BS22" s="105"/>
+      <c r="BT22" s="106"/>
     </row>
     <row r="23" spans="1:72" x14ac:dyDescent="0.25">
-      <c r="A23" s="76" t="s">
+      <c r="A23" s="73" t="s">
         <v>91</v>
       </c>
-      <c r="B23" s="77" t="s">
+      <c r="B23" s="74" t="s">
         <v>92</v>
       </c>
-      <c r="C23" s="78"/>
-      <c r="D23" s="78"/>
-      <c r="E23" s="77"/>
-      <c r="F23" s="77"/>
-      <c r="G23" s="77"/>
-      <c r="H23" s="77"/>
-      <c r="I23" s="79"/>
-      <c r="J23" s="80"/>
-      <c r="K23" s="81"/>
-      <c r="L23" s="81"/>
-      <c r="M23" s="82"/>
-      <c r="N23" s="82" t="str">
+      <c r="C23" s="75"/>
+      <c r="D23" s="75"/>
+      <c r="E23" s="74"/>
+      <c r="F23" s="74"/>
+      <c r="G23" s="74"/>
+      <c r="H23" s="74"/>
+      <c r="I23" s="76"/>
+      <c r="J23" s="77"/>
+      <c r="K23" s="78"/>
+      <c r="L23" s="78"/>
+      <c r="M23" s="79"/>
+      <c r="N23" s="79" t="str">
         <f>IF(OR(L23="",M23=""),"",L23-M23)</f>
         <v/>
       </c>
-      <c r="O23" s="80"/>
-      <c r="P23" s="81"/>
-      <c r="Q23" s="81"/>
-      <c r="R23" s="82"/>
-      <c r="S23" s="83" t="str">
+      <c r="O23" s="77"/>
+      <c r="P23" s="78"/>
+      <c r="Q23" s="78"/>
+      <c r="R23" s="79"/>
+      <c r="S23" s="80" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="T23" s="84"/>
-      <c r="U23" s="81"/>
-      <c r="V23" s="81"/>
-      <c r="W23" s="82"/>
-      <c r="X23" s="83" t="str">
+      <c r="T23" s="81"/>
+      <c r="U23" s="78"/>
+      <c r="V23" s="78"/>
+      <c r="W23" s="79"/>
+      <c r="X23" s="80" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="Y23" s="84"/>
-      <c r="Z23" s="81"/>
-      <c r="AA23" s="81"/>
-      <c r="AB23" s="82"/>
-      <c r="AC23" s="83" t="str">
+      <c r="Y23" s="81"/>
+      <c r="Z23" s="78"/>
+      <c r="AA23" s="78"/>
+      <c r="AB23" s="79"/>
+      <c r="AC23" s="80" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
-      <c r="AD23" s="84"/>
-      <c r="AE23" s="81"/>
-      <c r="AF23" s="81"/>
-      <c r="AG23" s="82"/>
-      <c r="AH23" s="83" t="str">
+      <c r="AD23" s="81"/>
+      <c r="AE23" s="78"/>
+      <c r="AF23" s="78"/>
+      <c r="AG23" s="79"/>
+      <c r="AH23" s="80" t="str">
         <f t="shared" si="17"/>
         <v/>
       </c>
-      <c r="AI23" s="84"/>
-      <c r="AJ23" s="81"/>
-      <c r="AK23" s="81"/>
-      <c r="AL23" s="82"/>
-      <c r="AM23" s="83" t="str">
+      <c r="AI23" s="81"/>
+      <c r="AJ23" s="78"/>
+      <c r="AK23" s="78"/>
+      <c r="AL23" s="79"/>
+      <c r="AM23" s="80" t="str">
         <f t="shared" si="18"/>
         <v/>
       </c>
-      <c r="AN23" s="84"/>
-      <c r="AO23" s="81"/>
-      <c r="AP23" s="81"/>
-      <c r="AQ23" s="82"/>
-      <c r="AR23" s="83" t="str">
+      <c r="AN23" s="81"/>
+      <c r="AO23" s="78"/>
+      <c r="AP23" s="78"/>
+      <c r="AQ23" s="79"/>
+      <c r="AR23" s="80" t="str">
         <f t="shared" si="19"/>
         <v/>
       </c>
-      <c r="AS23" s="84"/>
-      <c r="AT23" s="81"/>
-      <c r="AU23" s="81"/>
-      <c r="AV23" s="82"/>
-      <c r="AW23" s="83" t="str">
+      <c r="AS23" s="81"/>
+      <c r="AT23" s="78"/>
+      <c r="AU23" s="78"/>
+      <c r="AV23" s="79"/>
+      <c r="AW23" s="80" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="AX23" s="84"/>
-      <c r="AY23" s="81"/>
-      <c r="AZ23" s="81"/>
-      <c r="BA23" s="82"/>
-      <c r="BB23" s="83" t="str">
+      <c r="AX23" s="81"/>
+      <c r="AY23" s="78"/>
+      <c r="AZ23" s="78"/>
+      <c r="BA23" s="79"/>
+      <c r="BB23" s="80" t="str">
         <f t="shared" si="21"/>
         <v/>
       </c>
-      <c r="BC23" s="84"/>
-      <c r="BD23" s="81"/>
-      <c r="BE23" s="81"/>
-      <c r="BF23" s="82"/>
-      <c r="BG23" s="83" t="str">
+      <c r="BC23" s="81"/>
+      <c r="BD23" s="78"/>
+      <c r="BE23" s="78"/>
+      <c r="BF23" s="79"/>
+      <c r="BG23" s="80" t="str">
         <f t="shared" si="22"/>
         <v/>
       </c>
-      <c r="BH23" s="84"/>
-      <c r="BI23" s="81"/>
-      <c r="BJ23" s="81"/>
-      <c r="BK23" s="82"/>
-      <c r="BL23" s="83" t="str">
+      <c r="BH23" s="81"/>
+      <c r="BI23" s="78"/>
+      <c r="BJ23" s="78"/>
+      <c r="BK23" s="79"/>
+      <c r="BL23" s="80" t="str">
         <f t="shared" si="23"/>
         <v/>
       </c>
-      <c r="BM23" s="84"/>
-      <c r="BN23" s="81"/>
-      <c r="BO23" s="81"/>
-      <c r="BP23" s="82"/>
-      <c r="BQ23" s="83" t="str">
+      <c r="BM23" s="81"/>
+      <c r="BN23" s="78"/>
+      <c r="BO23" s="78"/>
+      <c r="BP23" s="79"/>
+      <c r="BQ23" s="80" t="str">
         <f t="shared" si="24"/>
         <v/>
       </c>
-      <c r="BR23" s="80">
+      <c r="BR23" s="77">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="BS23" s="85"/>
-      <c r="BT23" s="86"/>
+      <c r="BS23" s="82"/>
+      <c r="BT23" s="83"/>
     </row>
     <row r="24" spans="1:72" x14ac:dyDescent="0.25">
-      <c r="A24" s="87"/>
-      <c r="B24" s="88"/>
-      <c r="C24" s="89"/>
-      <c r="D24" s="89"/>
-      <c r="E24" s="88"/>
-      <c r="F24" s="88"/>
-      <c r="G24" s="88"/>
-      <c r="H24" s="88"/>
-      <c r="I24" s="90"/>
-      <c r="J24" s="91"/>
-      <c r="K24" s="92"/>
-      <c r="L24" s="92"/>
-      <c r="M24" s="52"/>
-      <c r="N24" s="52" t="str">
+      <c r="A24" s="84"/>
+      <c r="B24" s="85"/>
+      <c r="C24" s="86"/>
+      <c r="D24" s="86"/>
+      <c r="E24" s="85"/>
+      <c r="F24" s="85"/>
+      <c r="G24" s="85"/>
+      <c r="H24" s="85"/>
+      <c r="I24" s="87"/>
+      <c r="J24" s="88"/>
+      <c r="K24" s="89"/>
+      <c r="L24" s="89"/>
+      <c r="M24" s="50"/>
+      <c r="N24" s="50" t="str">
         <f t="shared" ref="N24:N25" si="25">IF(OR(L24="",M24=""),"",L24-M24)</f>
         <v/>
       </c>
-      <c r="O24" s="91"/>
-      <c r="P24" s="92"/>
-      <c r="Q24" s="92"/>
-      <c r="R24" s="52"/>
-      <c r="S24" s="53" t="str">
+      <c r="O24" s="88"/>
+      <c r="P24" s="89"/>
+      <c r="Q24" s="89"/>
+      <c r="R24" s="50"/>
+      <c r="S24" s="51" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="T24" s="58"/>
-      <c r="U24" s="92"/>
-      <c r="V24" s="92"/>
-      <c r="W24" s="52"/>
-      <c r="X24" s="53" t="str">
+      <c r="T24" s="56"/>
+      <c r="U24" s="89"/>
+      <c r="V24" s="89"/>
+      <c r="W24" s="50"/>
+      <c r="X24" s="51" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="Y24" s="58"/>
-      <c r="Z24" s="92"/>
-      <c r="AA24" s="92"/>
-      <c r="AB24" s="52"/>
-      <c r="AC24" s="53" t="str">
+      <c r="Y24" s="56"/>
+      <c r="Z24" s="89"/>
+      <c r="AA24" s="89"/>
+      <c r="AB24" s="50"/>
+      <c r="AC24" s="51" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
-      <c r="AD24" s="58"/>
-      <c r="AE24" s="92"/>
-      <c r="AF24" s="92"/>
-      <c r="AG24" s="52"/>
-      <c r="AH24" s="53" t="str">
+      <c r="AD24" s="56"/>
+      <c r="AE24" s="89"/>
+      <c r="AF24" s="89"/>
+      <c r="AG24" s="50"/>
+      <c r="AH24" s="51" t="str">
         <f t="shared" si="17"/>
         <v/>
       </c>
-      <c r="AI24" s="58"/>
-      <c r="AJ24" s="92"/>
-      <c r="AK24" s="92"/>
-      <c r="AL24" s="52"/>
-      <c r="AM24" s="53" t="str">
+      <c r="AI24" s="56"/>
+      <c r="AJ24" s="89"/>
+      <c r="AK24" s="89"/>
+      <c r="AL24" s="50"/>
+      <c r="AM24" s="51" t="str">
         <f t="shared" si="18"/>
         <v/>
       </c>
-      <c r="AN24" s="58"/>
-      <c r="AO24" s="92"/>
-      <c r="AP24" s="92"/>
-      <c r="AQ24" s="52"/>
-      <c r="AR24" s="53" t="str">
+      <c r="AN24" s="56"/>
+      <c r="AO24" s="89"/>
+      <c r="AP24" s="89"/>
+      <c r="AQ24" s="50"/>
+      <c r="AR24" s="51" t="str">
         <f t="shared" si="19"/>
         <v/>
       </c>
-      <c r="AS24" s="58"/>
-      <c r="AT24" s="92"/>
-      <c r="AU24" s="92"/>
-      <c r="AV24" s="52"/>
-      <c r="AW24" s="53" t="str">
+      <c r="AS24" s="56"/>
+      <c r="AT24" s="89"/>
+      <c r="AU24" s="89"/>
+      <c r="AV24" s="50"/>
+      <c r="AW24" s="51" t="str">
         <f t="shared" si="20"/>
         <v/>
       </c>
-      <c r="AX24" s="58"/>
-      <c r="AY24" s="92"/>
-      <c r="AZ24" s="92"/>
-      <c r="BA24" s="52"/>
-      <c r="BB24" s="53" t="str">
+      <c r="AX24" s="56"/>
+      <c r="AY24" s="89"/>
+      <c r="AZ24" s="89"/>
+      <c r="BA24" s="50"/>
+      <c r="BB24" s="51" t="str">
         <f t="shared" si="21"/>
         <v/>
       </c>
-      <c r="BC24" s="58"/>
-      <c r="BD24" s="92"/>
-      <c r="BE24" s="92"/>
-      <c r="BF24" s="52"/>
-      <c r="BG24" s="53" t="str">
+      <c r="BC24" s="56"/>
+      <c r="BD24" s="89"/>
+      <c r="BE24" s="89"/>
+      <c r="BF24" s="50"/>
+      <c r="BG24" s="51" t="str">
         <f t="shared" si="22"/>
         <v/>
       </c>
-      <c r="BH24" s="58"/>
-      <c r="BI24" s="92"/>
-      <c r="BJ24" s="92"/>
-      <c r="BK24" s="52"/>
-      <c r="BL24" s="53" t="str">
+      <c r="BH24" s="56"/>
+      <c r="BI24" s="89"/>
+      <c r="BJ24" s="89"/>
+      <c r="BK24" s="50"/>
+      <c r="BL24" s="51" t="str">
         <f t="shared" si="23"/>
         <v/>
       </c>
-      <c r="BM24" s="58"/>
-      <c r="BN24" s="92"/>
-      <c r="BO24" s="92"/>
-      <c r="BP24" s="52"/>
-      <c r="BQ24" s="53" t="str">
+      <c r="BM24" s="56"/>
+      <c r="BN24" s="89"/>
+      <c r="BO24" s="89"/>
+      <c r="BP24" s="50"/>
+      <c r="BQ24" s="51" t="str">
         <f t="shared" si="24"/>
         <v/>
       </c>
-      <c r="BR24" s="51">
+      <c r="BR24" s="49">
         <f t="shared" ref="BR24:BR25" si="26">SUM(IF(M24&lt;&gt;"",M24,IF(L24&lt;&gt;"",L24,K24)),IF(R24&lt;&gt;"",R24,IF(Q24&lt;&gt;"",Q24,P24)),IF(W24&lt;&gt;"",W24,IF(V24&lt;&gt;"",V24,U24)),IF(AB24&lt;&gt;"",AB24,IF(AA24&lt;&gt;"",AA24,Z24)),IF(AG24&lt;&gt;"",AG24,IF(AF24&lt;&gt;"",AF24,AE24)),IF(AL24&lt;&gt;"",AL24,IF(AK24&lt;&gt;"",AK24,AJ24)),IF(AQ24&lt;&gt;"",AQ24,IF(AP24&lt;&gt;"",AP24,AO24)),IF(AV24&lt;&gt;"",AV24,IF(AU24&lt;&gt;"",AU24,AT24)),IF(BA24&lt;&gt;"",BA24,IF(AZ24&lt;&gt;"",AZ24,AY24)),IF(BF24&lt;&gt;"",BF24,IF(BE24&lt;&gt;"",BE24,BD24)),IF(BK24&lt;&gt;"",BK24,IF(BJ24&lt;&gt;"",BJ24,BI24)),IF(BP24&lt;&gt;"",BP24,IF(BO24&lt;&gt;"",BO24,BN24)))</f>
         <v>0</v>
       </c>
-      <c r="BS24" s="93"/>
-      <c r="BT24" s="94"/>
+      <c r="BS24" s="90"/>
+      <c r="BT24" s="91"/>
     </row>
     <row r="25" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="59" t="s">
+      <c r="A25" s="57" t="s">
         <v>91</v>
       </c>
-      <c r="B25" s="60" t="s">
+      <c r="B25" s="58" t="s">
         <v>92</v>
       </c>
-      <c r="C25" s="95"/>
-      <c r="D25" s="95"/>
-      <c r="E25" s="60" t="s">
+      <c r="C25" s="92"/>
+      <c r="D25" s="92"/>
+      <c r="E25" s="58" t="s">
         <v>92</v>
       </c>
-      <c r="F25" s="60"/>
-      <c r="G25" s="60"/>
-      <c r="H25" s="60"/>
-      <c r="I25" s="61"/>
-      <c r="J25" s="66"/>
-      <c r="K25" s="62"/>
-      <c r="L25" s="62"/>
-      <c r="M25" s="63">
+      <c r="F25" s="58"/>
+      <c r="G25" s="58"/>
+      <c r="H25" s="58"/>
+      <c r="I25" s="59"/>
+      <c r="J25" s="64"/>
+      <c r="K25" s="60"/>
+      <c r="L25" s="60"/>
+      <c r="M25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=1,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),0)</f>
         <v>0</v>
       </c>
-      <c r="N25" s="96" t="str">
+      <c r="N25" s="93" t="str">
         <f t="shared" ca="1" si="25"/>
         <v/>
       </c>
-      <c r="O25" s="66"/>
-      <c r="P25" s="62"/>
-      <c r="Q25" s="62"/>
-      <c r="R25" s="63">
+      <c r="O25" s="64"/>
+      <c r="P25" s="60"/>
+      <c r="Q25" s="60"/>
+      <c r="R25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=2,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),0)</f>
         <v>0</v>
       </c>
-      <c r="S25" s="64"/>
-      <c r="T25" s="65"/>
-      <c r="U25" s="62"/>
-      <c r="V25" s="62"/>
-      <c r="W25" s="63">
+      <c r="S25" s="62"/>
+      <c r="T25" s="63"/>
+      <c r="U25" s="60"/>
+      <c r="V25" s="60"/>
+      <c r="W25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=3,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),0)</f>
         <v>0</v>
       </c>
-      <c r="X25" s="64"/>
-      <c r="Y25" s="65"/>
-      <c r="Z25" s="62"/>
-      <c r="AA25" s="62"/>
-      <c r="AB25" s="63">
+      <c r="X25" s="62"/>
+      <c r="Y25" s="63"/>
+      <c r="Z25" s="60"/>
+      <c r="AA25" s="60"/>
+      <c r="AB25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=4,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),0)</f>
         <v>0</v>
       </c>
-      <c r="AC25" s="64"/>
-      <c r="AD25" s="65"/>
-      <c r="AE25" s="62"/>
-      <c r="AF25" s="62"/>
-      <c r="AG25" s="63">
+      <c r="AC25" s="62"/>
+      <c r="AD25" s="63"/>
+      <c r="AE25" s="60"/>
+      <c r="AF25" s="60"/>
+      <c r="AG25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=5,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),0)</f>
         <v>0</v>
       </c>
-      <c r="AH25" s="64"/>
-      <c r="AI25" s="65"/>
-      <c r="AJ25" s="62"/>
-      <c r="AK25" s="62"/>
-      <c r="AL25" s="63">
+      <c r="AH25" s="62"/>
+      <c r="AI25" s="63"/>
+      <c r="AJ25" s="60"/>
+      <c r="AK25" s="60"/>
+      <c r="AL25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=6,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),0)</f>
         <v>0</v>
       </c>
-      <c r="AM25" s="64"/>
-      <c r="AN25" s="65"/>
-      <c r="AO25" s="62"/>
-      <c r="AP25" s="62"/>
-      <c r="AQ25" s="63">
+      <c r="AM25" s="62"/>
+      <c r="AN25" s="63"/>
+      <c r="AO25" s="60"/>
+      <c r="AP25" s="60"/>
+      <c r="AQ25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=7,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),0)</f>
         <v>0</v>
       </c>
-      <c r="AR25" s="64"/>
-      <c r="AS25" s="65"/>
-      <c r="AT25" s="62"/>
-      <c r="AU25" s="62"/>
-      <c r="AV25" s="63">
+      <c r="AR25" s="62"/>
+      <c r="AS25" s="63"/>
+      <c r="AT25" s="60"/>
+      <c r="AU25" s="60"/>
+      <c r="AV25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=8,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),0)</f>
         <v>0</v>
       </c>
-      <c r="AW25" s="64"/>
-      <c r="AX25" s="65"/>
-      <c r="AY25" s="62"/>
-      <c r="AZ25" s="62"/>
-      <c r="BA25" s="63">
+      <c r="AW25" s="62"/>
+      <c r="AX25" s="63"/>
+      <c r="AY25" s="60"/>
+      <c r="AZ25" s="60"/>
+      <c r="BA25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=9,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),0)</f>
         <v>0</v>
       </c>
-      <c r="BB25" s="64"/>
-      <c r="BC25" s="65"/>
-      <c r="BD25" s="62"/>
-      <c r="BE25" s="62"/>
-      <c r="BF25" s="63">
+      <c r="BB25" s="62"/>
+      <c r="BC25" s="63"/>
+      <c r="BD25" s="60"/>
+      <c r="BE25" s="60"/>
+      <c r="BF25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=10,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),0)</f>
         <v>0</v>
       </c>
-      <c r="BG25" s="64"/>
-      <c r="BH25" s="65"/>
-      <c r="BI25" s="62"/>
-      <c r="BJ25" s="62"/>
-      <c r="BK25" s="63">
+      <c r="BG25" s="62"/>
+      <c r="BH25" s="63"/>
+      <c r="BI25" s="60"/>
+      <c r="BJ25" s="60"/>
+      <c r="BK25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;=11,($BS$13-$BR$13)/(12-(MONTH(TODAY()) + 1)),IF(MONTH(TODAY())=11,($BS$13-$BR$13)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="BL25" s="64"/>
-      <c r="BM25" s="65"/>
-      <c r="BN25" s="62"/>
-      <c r="BO25" s="62"/>
-      <c r="BP25" s="63">
+      <c r="BL25" s="62"/>
+      <c r="BM25" s="63"/>
+      <c r="BN25" s="60"/>
+      <c r="BO25" s="60"/>
+      <c r="BP25" s="61">
         <f ca="1">IF((MONTH(TODAY()) + 2)&lt;12,($BS$13-$BR$13)/(12-(MONTH(TODAY())+ 1)),IF(MONTH(TODAY())=11,($BS$13-$BR$13)/2,IF(OR(MONTH(TODAY())=10,MONTH(TODAY())=12),($BS$13-$BR$13),0)))</f>
         <v>0</v>
       </c>
-      <c r="BQ25" s="64"/>
-      <c r="BR25" s="66">
+      <c r="BQ25" s="62"/>
+      <c r="BR25" s="64">
         <f t="shared" ca="1" si="26"/>
         <v>0</v>
       </c>
-      <c r="BS25" s="97"/>
-      <c r="BT25" s="98"/>
+      <c r="BS25" s="94"/>
+      <c r="BT25" s="95"/>
     </row>
     <row r="26" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -3764,6 +3837,29 @@
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="BM11:BQ11"/>
+    <mergeCell ref="BM13:BQ13"/>
+    <mergeCell ref="O11:S11"/>
+    <mergeCell ref="J11:N11"/>
+    <mergeCell ref="T11:X11"/>
+    <mergeCell ref="Y11:AC11"/>
+    <mergeCell ref="AD11:AH11"/>
+    <mergeCell ref="AI11:AM11"/>
+    <mergeCell ref="AN11:AR11"/>
+    <mergeCell ref="AS11:AW11"/>
+    <mergeCell ref="AX11:BB11"/>
+    <mergeCell ref="BC11:BG11"/>
+    <mergeCell ref="BH11:BL11"/>
+    <mergeCell ref="O13:S13"/>
+    <mergeCell ref="J13:N13"/>
+    <mergeCell ref="T13:X13"/>
+    <mergeCell ref="BC12:BG12"/>
+    <mergeCell ref="BH12:BL12"/>
+    <mergeCell ref="Y13:AC13"/>
+    <mergeCell ref="AD13:AH13"/>
+    <mergeCell ref="AI13:AM13"/>
+    <mergeCell ref="AN13:AR13"/>
+    <mergeCell ref="AS13:AW13"/>
     <mergeCell ref="BM12:BQ12"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="H12:I12"/>
@@ -3780,29 +3876,6 @@
     <mergeCell ref="AN12:AR12"/>
     <mergeCell ref="AS12:AW12"/>
     <mergeCell ref="AX12:BB12"/>
-    <mergeCell ref="BC12:BG12"/>
-    <mergeCell ref="BH12:BL12"/>
-    <mergeCell ref="Y13:AC13"/>
-    <mergeCell ref="AD13:AH13"/>
-    <mergeCell ref="AI13:AM13"/>
-    <mergeCell ref="AN13:AR13"/>
-    <mergeCell ref="AS13:AW13"/>
-    <mergeCell ref="BM11:BQ11"/>
-    <mergeCell ref="BM13:BQ13"/>
-    <mergeCell ref="O11:S11"/>
-    <mergeCell ref="J11:N11"/>
-    <mergeCell ref="T11:X11"/>
-    <mergeCell ref="Y11:AC11"/>
-    <mergeCell ref="AD11:AH11"/>
-    <mergeCell ref="AI11:AM11"/>
-    <mergeCell ref="AN11:AR11"/>
-    <mergeCell ref="AS11:AW11"/>
-    <mergeCell ref="AX11:BB11"/>
-    <mergeCell ref="BC11:BG11"/>
-    <mergeCell ref="BH11:BL11"/>
-    <mergeCell ref="O13:S13"/>
-    <mergeCell ref="J13:N13"/>
-    <mergeCell ref="T13:X13"/>
   </mergeCells>
   <conditionalFormatting sqref="M15:M24 R15:R24 W15:W24 AB15:AB24 AG15:AG24 AL15:AL24 AQ15:AQ24 AV15:AV24 BA15:BA24 BF15:BF24 BK15:BK24 BP15:BP24">
     <cfRule type="expression" dxfId="7" priority="8">
@@ -3851,14 +3924,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19b1ad6d-7bbd-4338-adb0-a51e11e836c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4099,27 +4170,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19b1ad6d-7bbd-4338-adb0-a51e11e836c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BC2B212-31BA-49FB-B215-9E14B2C60948}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="19b1ad6d-7bbd-4338-adb0-a51e11e836c7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4144,9 +4208,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BC2B212-31BA-49FB-B215-9E14B2C60948}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="19b1ad6d-7bbd-4338-adb0-a51e11e836c7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>